<commit_message>
reports: refresh consolidated reports (2026-06-11 batch re-run)
Re-run with all scenarios enabled, per-segment risk targets
(known 2.0 / new 4.0), RI optimizer disabled for new (real RI
uplifts, avg 1.64x), and the corrected rejection-rate basis:
rejections / through-the-door demand, canceled never a rejection.
Actual rejection rate is now scenario-invariant (known 41.98%,
new 50.54%) — definitional change vs the previously committed
reports, the portfolio itself is unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 10 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260610T184656Z_9d9e462ec54a  |  git 9d9e462ec54a (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T204933Z_2f5e5c364e7d  |  git 2f5e5c364e7d (dirty)  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>70.8%</t>
+          <t>44.5%</t>
         </is>
       </c>
       <c r="H4" s="5" t="n"/>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>67.7%</t>
+          <t>39.3%</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
@@ -1574,10 +1574,10 @@
         <v>-0.6405099999999999</v>
       </c>
       <c r="K32" s="23" t="n">
-        <v>74.24233792276243</v>
+        <v>49.40800991602669</v>
       </c>
       <c r="L32" s="23" t="n">
-        <v>72.39013709994427</v>
+        <v>46.76757379914275</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
@@ -1618,10 +1618,10 @@
         <v>-0.1628530000000001</v>
       </c>
       <c r="K33" s="23" t="n">
-        <v>74.02054301856376</v>
+        <v>49.40800991602669</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>70.84831063154357</v>
+        <v>44.46941954207335</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
@@ -1662,10 +1662,10 @@
         <v>0.2944300000000002</v>
       </c>
       <c r="K34" s="23" t="n">
-        <v>73.81244128259937</v>
+        <v>49.40800991602669</v>
       </c>
       <c r="L34" s="23" t="n">
-        <v>69.79869537118483</v>
+        <v>42.77193076841708</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -1706,10 +1706,10 @@
         <v>-0.4682839999999997</v>
       </c>
       <c r="K35" s="23" t="n">
-        <v>71.18716767463916</v>
+        <v>44.00757330718467</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>70.02310323686397</v>
+        <v>41.79545881864378</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
@@ -1750,10 +1750,10 @@
         <v>0.01875000000000027</v>
       </c>
       <c r="K36" s="23" t="n">
-        <v>70.56801302481421</v>
+        <v>44.00757330718467</v>
       </c>
       <c r="L36" s="23" t="n">
-        <v>67.66133606426843</v>
+        <v>39.31302155563219</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
@@ -1794,10 +1794,10 @@
         <v>0.4820120000000001</v>
       </c>
       <c r="K37" s="23" t="n">
-        <v>70.05429556473032</v>
+        <v>44.00757330718467</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>66.14746868782397</v>
+        <v>37.76882116610484</v>
       </c>
     </row>
     <row r="38"/>
@@ -1867,7 +1867,7 @@
         <v>-0.1760220000000001</v>
       </c>
       <c r="G41" s="28" t="n">
-        <v>74.13439358022929</v>
+        <v>45.51050494280762</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
@@ -1892,7 +1892,7 @@
         <v>-0.143348</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>52.69986400691571</v>
+        <v>37.66285234135594</v>
       </c>
     </row>
     <row r="43"/>
@@ -1962,7 +1962,7 @@
         <v>0.04153899999999977</v>
       </c>
       <c r="G46" s="33" t="n">
-        <v>71.10119487142701</v>
+        <v>40.49204046882839</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
@@ -1987,7 +1987,7 @@
         <v>-0.06094500000000003</v>
       </c>
       <c r="G47" s="28" t="n">
-        <v>46.86633947340729</v>
+        <v>31.02871271964337</v>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260610T184656Z_9d9e462ec54a  ·  git 9d9e462ec54a (dirty)  ·  cfg 341cb26ac9bc</t>
+          <t>20260611T204933Z_2f5e5c364e7d  ·  git 2f5e5c364e7d (dirty)  ·  cfg 013888af7168</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>56.32057180816309</v>
+        <v>41.98258608500487</v>
       </c>
       <c r="F5" s="25" t="inlineStr"/>
       <c r="G5" s="25" t="inlineStr"/>
@@ -5341,7 +5341,7 @@
         <v>1.082892747252677</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>52.69986400691571</v>
+        <v>37.66285234135594</v>
       </c>
       <c r="F8" s="59" t="n">
         <v>29420298.83583964</v>
@@ -5518,7 +5518,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>49.38800136401866</v>
+        <v>33.80033360243112</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>1.088158</v>
@@ -5578,7 +5578,7 @@
         <v>1.049823400746294</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>46.86633947340729</v>
+        <v>31.02871271964337</v>
       </c>
       <c r="F8" s="58" t="n">
         <v>0.955581</v>
@@ -5795,7 +5795,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>77.2254219147992</v>
+        <v>50.54375134291313</v>
       </c>
       <c r="F5" s="25" t="inlineStr"/>
       <c r="G5" s="25" t="inlineStr"/>
@@ -5911,7 +5911,7 @@
         <v>1.135722748540335</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>74.13439358022929</v>
+        <v>45.51050494280762</v>
       </c>
       <c r="F8" s="59" t="n">
         <v>87983684.34945849</v>
@@ -6088,7 +6088,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>74.07156010782394</v>
+        <v>45.46026283164456</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>2.527868</v>
@@ -6148,7 +6148,7 @@
         <v>1.114560121964501</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>71.10119487142701</v>
+        <v>40.49204046882839</v>
       </c>
       <c r="F8" s="58" t="n">
         <v>2.408918</v>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (2026-06-11 batch re-run) (#109)
Re-run with all scenarios enabled, per-segment risk targets
(known 2.0 / new 4.0), RI optimizer disabled for new (real RI
uplifts, avg 1.64x), and the corrected rejection-rate basis:
rejections / through-the-door demand, canceled never a rejection.
Actual rejection rate is now scenario-invariant (known 41.98%,
new 50.54%) — definitional change vs the previously committed
reports, the portfolio itself is unchanged.

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 10 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260610T184656Z_9d9e462ec54a  |  git 9d9e462ec54a (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T204933Z_2f5e5c364e7d  |  git 2f5e5c364e7d (dirty)  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>70.8%</t>
+          <t>44.5%</t>
         </is>
       </c>
       <c r="H4" s="5" t="n"/>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>67.7%</t>
+          <t>39.3%</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
@@ -1574,10 +1574,10 @@
         <v>-0.6405099999999999</v>
       </c>
       <c r="K32" s="23" t="n">
-        <v>74.24233792276243</v>
+        <v>49.40800991602669</v>
       </c>
       <c r="L32" s="23" t="n">
-        <v>72.39013709994427</v>
+        <v>46.76757379914275</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
@@ -1618,10 +1618,10 @@
         <v>-0.1628530000000001</v>
       </c>
       <c r="K33" s="23" t="n">
-        <v>74.02054301856376</v>
+        <v>49.40800991602669</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>70.84831063154357</v>
+        <v>44.46941954207335</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
@@ -1662,10 +1662,10 @@
         <v>0.2944300000000002</v>
       </c>
       <c r="K34" s="23" t="n">
-        <v>73.81244128259937</v>
+        <v>49.40800991602669</v>
       </c>
       <c r="L34" s="23" t="n">
-        <v>69.79869537118483</v>
+        <v>42.77193076841708</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -1706,10 +1706,10 @@
         <v>-0.4682839999999997</v>
       </c>
       <c r="K35" s="23" t="n">
-        <v>71.18716767463916</v>
+        <v>44.00757330718467</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>70.02310323686397</v>
+        <v>41.79545881864378</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
@@ -1750,10 +1750,10 @@
         <v>0.01875000000000027</v>
       </c>
       <c r="K36" s="23" t="n">
-        <v>70.56801302481421</v>
+        <v>44.00757330718467</v>
       </c>
       <c r="L36" s="23" t="n">
-        <v>67.66133606426843</v>
+        <v>39.31302155563219</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
@@ -1794,10 +1794,10 @@
         <v>0.4820120000000001</v>
       </c>
       <c r="K37" s="23" t="n">
-        <v>70.05429556473032</v>
+        <v>44.00757330718467</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>66.14746868782397</v>
+        <v>37.76882116610484</v>
       </c>
     </row>
     <row r="38"/>
@@ -1867,7 +1867,7 @@
         <v>-0.1760220000000001</v>
       </c>
       <c r="G41" s="28" t="n">
-        <v>74.13439358022929</v>
+        <v>45.51050494280762</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
@@ -1892,7 +1892,7 @@
         <v>-0.143348</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>52.69986400691571</v>
+        <v>37.66285234135594</v>
       </c>
     </row>
     <row r="43"/>
@@ -1962,7 +1962,7 @@
         <v>0.04153899999999977</v>
       </c>
       <c r="G46" s="33" t="n">
-        <v>71.10119487142701</v>
+        <v>40.49204046882839</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
@@ -1987,7 +1987,7 @@
         <v>-0.06094500000000003</v>
       </c>
       <c r="G47" s="28" t="n">
-        <v>46.86633947340729</v>
+        <v>31.02871271964337</v>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260610T184656Z_9d9e462ec54a  ·  git 9d9e462ec54a (dirty)  ·  cfg 341cb26ac9bc</t>
+          <t>20260611T204933Z_2f5e5c364e7d  ·  git 2f5e5c364e7d (dirty)  ·  cfg 013888af7168</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>56.32057180816309</v>
+        <v>41.98258608500487</v>
       </c>
       <c r="F5" s="25" t="inlineStr"/>
       <c r="G5" s="25" t="inlineStr"/>
@@ -5341,7 +5341,7 @@
         <v>1.082892747252677</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>52.69986400691571</v>
+        <v>37.66285234135594</v>
       </c>
       <c r="F8" s="59" t="n">
         <v>29420298.83583964</v>
@@ -5518,7 +5518,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>49.38800136401866</v>
+        <v>33.80033360243112</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>1.088158</v>
@@ -5578,7 +5578,7 @@
         <v>1.049823400746294</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>46.86633947340729</v>
+        <v>31.02871271964337</v>
       </c>
       <c r="F8" s="58" t="n">
         <v>0.955581</v>
@@ -5795,7 +5795,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>77.2254219147992</v>
+        <v>50.54375134291313</v>
       </c>
       <c r="F5" s="25" t="inlineStr"/>
       <c r="G5" s="25" t="inlineStr"/>
@@ -5911,7 +5911,7 @@
         <v>1.135722748540335</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>74.13439358022929</v>
+        <v>45.51050494280762</v>
       </c>
       <c r="F8" s="59" t="n">
         <v>87983684.34945849</v>
@@ -6088,7 +6088,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>74.07156010782394</v>
+        <v>45.46026283164456</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>2.527868</v>
@@ -6148,7 +6148,7 @@
         <v>1.114560121964501</v>
       </c>
       <c r="E8" s="58" t="n">
-        <v>71.10119487142701</v>
+        <v>40.49204046882839</v>
       </c>
       <c r="F8" s="58" t="n">
         <v>2.408918</v>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (2026-06-15 batch re-run)
Regenerated from a full batch run on the current data with the
oa_amt_h0-weighted prediction-surface markers (#110).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T204933Z_2f5e5c364e7d  |  git 2f5e5c364e7d (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T214313Z_7a9403db5573  |  git 7a9403db5573  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260611T204933Z_2f5e5c364e7d  ·  git 2f5e5c364e7d (dirty)  ·  cfg 013888af7168</t>
+          <t>20260611T214313Z_7a9403db5573  ·  git 7a9403db5573  ·  cfg 013888af7168</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (2026-06-15 batch re-run) (#112)
Regenerated from a full batch run on the current data with the
oa_amt_h0-weighted prediction-surface markers (#110).

Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T204933Z_2f5e5c364e7d  |  git 2f5e5c364e7d (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T214313Z_7a9403db5573  |  git 7a9403db5573  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260611T204933Z_2f5e5c364e7d  ·  git 2f5e5c364e7d (dirty)  ·  cfg 013888af7168</t>
+          <t>20260611T214313Z_7a9403db5573  ·  git 7a9403db5573  ·  cfg 013888af7168</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (2026-06-15 re-run on sklearn 1.9.0 stack)
Regenerated from a full batch run on the upgraded dependency stack
(scikit-learn 1.9.0, matplotlib 3.11.0, plotly 6.8.0; #113). A full
cell-by-cell comparison across all 7 sheets vs the prior reports shows
only 2 differing cells, both provenance (generated date + run-id/git);
every numeric/content cell is bit-identical. Confirms the dependency
bump is behavior-neutral for headline risk/production and cutoffs.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T214313Z_7a9403db5573  |  git 7a9403db5573  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 15 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260615T193455Z_505a36897707  |  git 505a36897707  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260611T214313Z_7a9403db5573  ·  git 7a9403db5573  ·  cfg 013888af7168</t>
+          <t>20260615T193455Z_505a36897707  ·  git 505a36897707  ·  cfg 013888af7168</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (2026-06-15 re-run on sklearn 1.9.0 stack) (#114)
Regenerated from a full batch run on the upgraded dependency stack
(scikit-learn 1.9.0, matplotlib 3.11.0, plotly 6.8.0; #113). A full
cell-by-cell comparison across all 7 sheets vs the prior reports shows
only 2 differing cells, both provenance (generated date + run-id/git);
every numeric/content cell is bit-identical. Confirms the dependency
bump is behavior-neutral for headline risk/production and cutoffs.

Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 11 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260611T214313Z_7a9403db5573  |  git 7a9403db5573  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 15 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260615T193455Z_505a36897707  |  git 505a36897707  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260611T214313Z_7a9403db5573  ·  git 7a9403db5573  ·  cfg 013888af7168</t>
+          <t>20260615T193455Z_505a36897707  ·  git 505a36897707  ·  cfg 013888af7168</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(reporting): make System Rejection Rate visible in Excel Exec Summary
Follow-up to #117. The System Rejection Rate KPI card landed as the far-right
5th card (column I), off-screen for most users — it read as "missing from the
Excel". And the "Scenario Overview — Total Portfolio" table showed the
production-basis rejection rate but not the system one.

- Reorder the Exec Summary KPI cards (Main + MR) to Production / Risk /
  Rejection Rate / System Rejection Rate / Production Delta, so the two
  rejection metrics sit side by side at columns E and G (in view); the derived
  Production Delta moves to the right.
- Add Actual + Optimum System Rejection Rate to the Scenario Overview table
  (now 14 cols) — it's now in every Exec Summary table that shows rejection
  rate (KPI cards, Scenario Overview, Top Segment Opportunities).

Excel-layout only; values/HTML unchanged. Regenerated reports included.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -404,10 +404,10 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -922,18 +922,18 @@
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="29" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 16 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260616T081716Z_3edc135c43ad  |  git 3edc135c43ad (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 16 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260616T091540Z_0d20a14a6fab  |  git 0d20a14a6fab  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -978,36 +978,36 @@
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>€+12,980,590</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>+12.2%</t>
+          <t>-0.16 pp</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>3.49%</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>-0.16 pp</t>
-        </is>
-      </c>
+          <t>44.5%</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>44.5%</t>
+          <t>42.3%</t>
         </is>
       </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>42.3%</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="n"/>
+          <t>€+12,980,590</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>+12.2%</t>
+        </is>
+      </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
           <t>MAIN PERIOD</t>
@@ -1023,25 +1023,25 @@
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Production Delta</t>
+          <t>Optimum Risk   95% CI [3.35–3.62]</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Optimum Risk   95% CI [3.35–3.62]</t>
+          <t>Rejection Rate</t>
         </is>
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Rejection Rate</t>
+          <t>System Rejection Rate</t>
         </is>
       </c>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>System Rejection Rate</t>
+          <t>Production Delta</t>
         </is>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -1055,36 +1055,36 @@
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>€+13,812,886</t>
+          <t>3.53%</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>+9.9%</t>
+          <t>+0.02 pp</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>3.53%</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>+0.02 pp</t>
-        </is>
-      </c>
+          <t>39.3%</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="n"/>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>37.0%</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="n"/>
+          <t>€+13,812,886</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>+9.9%</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
           <t>MR PERIOD</t>
@@ -1100,25 +1100,25 @@
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>MR Prod. Delta</t>
+          <t>MR Optimum Risk</t>
         </is>
       </c>
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>MR Optimum Risk</t>
+          <t>MR Rejection Rate</t>
         </is>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>MR Rejection Rate</t>
+          <t>MR System Rejection Rate</t>
         </is>
       </c>
       <c r="H7" s="10" t="n"/>
       <c r="I7" s="14" t="inlineStr">
         <is>
-          <t>MR System Rejection Rate</t>
+          <t>MR Prod. Delta</t>
         </is>
       </c>
       <c r="J7" s="10" t="n"/>
@@ -1559,6 +1559,16 @@
           <t>Optimum Rejection Rate (%)</t>
         </is>
       </c>
+      <c r="M31" s="18" t="inlineStr">
+        <is>
+          <t>Actual System Rejection Rate (%)</t>
+        </is>
+      </c>
+      <c r="N31" s="18" t="inlineStr">
+        <is>
+          <t>Optimum System Rejection Rate (%)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -1603,6 +1613,12 @@
       <c r="L32" s="23" t="n">
         <v>46.76757379914275</v>
       </c>
+      <c r="M32" s="23" t="n">
+        <v>47.19130464011302</v>
+      </c>
+      <c r="N32" s="23" t="n">
+        <v>44.72320719393468</v>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="19" t="inlineStr">
@@ -1647,6 +1663,12 @@
       <c r="L33" s="23" t="n">
         <v>44.46941954207335</v>
       </c>
+      <c r="M33" s="23" t="n">
+        <v>47.19130464011302</v>
+      </c>
+      <c r="N33" s="23" t="n">
+        <v>42.3272188245023</v>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
@@ -1691,6 +1713,12 @@
       <c r="L34" s="23" t="n">
         <v>42.77193076841708</v>
       </c>
+      <c r="M34" s="23" t="n">
+        <v>47.19130464011302</v>
+      </c>
+      <c r="N34" s="23" t="n">
+        <v>40.56074134462235</v>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
@@ -1735,6 +1763,12 @@
       <c r="L35" s="23" t="n">
         <v>41.79545881864378</v>
       </c>
+      <c r="M35" s="23" t="n">
+        <v>41.6561394100917</v>
+      </c>
+      <c r="N35" s="23" t="n">
+        <v>39.45831166587732</v>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="19" t="inlineStr">
@@ -1779,6 +1813,12 @@
       <c r="L36" s="23" t="n">
         <v>39.31302155563219</v>
       </c>
+      <c r="M36" s="23" t="n">
+        <v>41.6561394100917</v>
+      </c>
+      <c r="N36" s="23" t="n">
+        <v>36.95391118572438</v>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
@@ -1822,6 +1862,12 @@
       </c>
       <c r="L37" s="23" t="n">
         <v>37.76882116610484</v>
+      </c>
+      <c r="M37" s="23" t="n">
+        <v>41.6561394100917</v>
+      </c>
+      <c r="N37" s="23" t="n">
+        <v>35.4109004113693</v>
       </c>
     </row>
     <row r="38"/>
@@ -4320,7 +4366,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A30:L30"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A64:L64"/>
     <mergeCell ref="A10:L10"/>
@@ -4328,6 +4373,7 @@
     <mergeCell ref="A11:L11"/>
     <mergeCell ref="A49:L49"/>
     <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A30:N30"/>
     <mergeCell ref="A13:L13"/>
     <mergeCell ref="A14:L14"/>
     <mergeCell ref="A44:H44"/>
@@ -4434,7 +4480,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260616T081716Z_3edc135c43ad  ·  git 3edc135c43ad (dirty)  ·  cfg 013888af7168</t>
+          <t>20260616T091540Z_0d20a14a6fab  ·  git 0d20a14a6fab  ·  cfg 341cb26ac9bc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(reporting): make System Rejection Rate visible in Excel Exec Summary (#118)
Follow-up to #117. The System Rejection Rate KPI card landed as the far-right
5th card (column I), off-screen for most users — it read as "missing from the
Excel". And the "Scenario Overview — Total Portfolio" table showed the
production-basis rejection rate but not the system one.

- Reorder the Exec Summary KPI cards (Main + MR) to Production / Risk /
  Rejection Rate / System Rejection Rate / Production Delta, so the two
  rejection metrics sit side by side at columns E and G (in view); the derived
  Production Delta moves to the right.
- Add Actual + Optimum System Rejection Rate to the Scenario Overview table
  (now 14 cols) — it's now in every Exec Summary table that shows rejection
  rate (KPI cards, Scenario Overview, Top Segment Opportunities).

Excel-layout only; values/HTML unchanged. Regenerated reports included.

Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -404,10 +404,10 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -922,18 +922,18 @@
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="29" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
@@ -953,7 +953,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 16 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260616T081716Z_3edc135c43ad  |  git 3edc135c43ad (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 16 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260616T091540Z_0d20a14a6fab  |  git 0d20a14a6fab  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -978,36 +978,36 @@
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>€+12,980,590</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>+12.2%</t>
+          <t>-0.16 pp</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>3.49%</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>-0.16 pp</t>
-        </is>
-      </c>
+          <t>44.5%</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>44.5%</t>
+          <t>42.3%</t>
         </is>
       </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>42.3%</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="n"/>
+          <t>€+12,980,590</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>+12.2%</t>
+        </is>
+      </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
           <t>MAIN PERIOD</t>
@@ -1023,25 +1023,25 @@
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Production Delta</t>
+          <t>Optimum Risk   95% CI [3.35–3.62]</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Optimum Risk   95% CI [3.35–3.62]</t>
+          <t>Rejection Rate</t>
         </is>
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Rejection Rate</t>
+          <t>System Rejection Rate</t>
         </is>
       </c>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>System Rejection Rate</t>
+          <t>Production Delta</t>
         </is>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -1055,36 +1055,36 @@
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>€+13,812,886</t>
+          <t>3.53%</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>+9.9%</t>
+          <t>+0.02 pp</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>3.53%</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>+0.02 pp</t>
-        </is>
-      </c>
+          <t>39.3%</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="n"/>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>37.0%</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="n"/>
+          <t>€+13,812,886</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>+9.9%</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
           <t>MR PERIOD</t>
@@ -1100,25 +1100,25 @@
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>MR Prod. Delta</t>
+          <t>MR Optimum Risk</t>
         </is>
       </c>
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>MR Optimum Risk</t>
+          <t>MR Rejection Rate</t>
         </is>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>MR Rejection Rate</t>
+          <t>MR System Rejection Rate</t>
         </is>
       </c>
       <c r="H7" s="10" t="n"/>
       <c r="I7" s="14" t="inlineStr">
         <is>
-          <t>MR System Rejection Rate</t>
+          <t>MR Prod. Delta</t>
         </is>
       </c>
       <c r="J7" s="10" t="n"/>
@@ -1559,6 +1559,16 @@
           <t>Optimum Rejection Rate (%)</t>
         </is>
       </c>
+      <c r="M31" s="18" t="inlineStr">
+        <is>
+          <t>Actual System Rejection Rate (%)</t>
+        </is>
+      </c>
+      <c r="N31" s="18" t="inlineStr">
+        <is>
+          <t>Optimum System Rejection Rate (%)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -1603,6 +1613,12 @@
       <c r="L32" s="23" t="n">
         <v>46.76757379914275</v>
       </c>
+      <c r="M32" s="23" t="n">
+        <v>47.19130464011302</v>
+      </c>
+      <c r="N32" s="23" t="n">
+        <v>44.72320719393468</v>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="19" t="inlineStr">
@@ -1647,6 +1663,12 @@
       <c r="L33" s="23" t="n">
         <v>44.46941954207335</v>
       </c>
+      <c r="M33" s="23" t="n">
+        <v>47.19130464011302</v>
+      </c>
+      <c r="N33" s="23" t="n">
+        <v>42.3272188245023</v>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
@@ -1691,6 +1713,12 @@
       <c r="L34" s="23" t="n">
         <v>42.77193076841708</v>
       </c>
+      <c r="M34" s="23" t="n">
+        <v>47.19130464011302</v>
+      </c>
+      <c r="N34" s="23" t="n">
+        <v>40.56074134462235</v>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
@@ -1735,6 +1763,12 @@
       <c r="L35" s="23" t="n">
         <v>41.79545881864378</v>
       </c>
+      <c r="M35" s="23" t="n">
+        <v>41.6561394100917</v>
+      </c>
+      <c r="N35" s="23" t="n">
+        <v>39.45831166587732</v>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="19" t="inlineStr">
@@ -1779,6 +1813,12 @@
       <c r="L36" s="23" t="n">
         <v>39.31302155563219</v>
       </c>
+      <c r="M36" s="23" t="n">
+        <v>41.6561394100917</v>
+      </c>
+      <c r="N36" s="23" t="n">
+        <v>36.95391118572438</v>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
@@ -1822,6 +1862,12 @@
       </c>
       <c r="L37" s="23" t="n">
         <v>37.76882116610484</v>
+      </c>
+      <c r="M37" s="23" t="n">
+        <v>41.6561394100917</v>
+      </c>
+      <c r="N37" s="23" t="n">
+        <v>35.4109004113693</v>
       </c>
     </row>
     <row r="38"/>
@@ -4320,7 +4366,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A30:L30"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A64:L64"/>
     <mergeCell ref="A10:L10"/>
@@ -4328,6 +4373,7 @@
     <mergeCell ref="A11:L11"/>
     <mergeCell ref="A49:L49"/>
     <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A30:N30"/>
     <mergeCell ref="A13:L13"/>
     <mergeCell ref="A14:L14"/>
     <mergeCell ref="A44:H44"/>
@@ -4434,7 +4480,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260616T081716Z_3edc135c43ad  ·  git 3edc135c43ad (dirty)  ·  cfg 013888af7168</t>
+          <t>20260616T091540Z_0d20a14a6fab  ·  git 0d20a14a6fab  ·  cfg 341cb26ac9bc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (K=12 octroi binning)
Regenerated after adopting the K=12 fixed octroi grid + retraining. Consolidated
base risk 3.65% -> 3.45%; known on a 20x12 grid, new fixed-cutoffs on 12x20.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -920,7 +920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U87"/>
+  <dimension ref="A1:U89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -932,7 +932,7 @@
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="29" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
@@ -956,7 +956,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 17 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260617T085641Z_b53c771578b7  |  git b53c771578b7 (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 17 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260617T114353Z_b1bd4685bfc4  |  git b1bd4685bfc4 (dirty)  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -975,18 +975,18 @@
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>€118,931,141</t>
+          <t>€118,820,800</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>-0.21 pp</t>
+          <t>-0.20 pp</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -997,18 +997,18 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>42.5%</t>
+          <t>42.6%</t>
         </is>
       </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>€+12,624,715</t>
+          <t>€+12,514,374</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>+11.9%</t>
+          <t>+11.8%</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -1020,13 +1020,13 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Optimum Production   95% CI [€118.6M–€119.3M]</t>
+          <t>Optimum Production   95% CI [€118.5M–€119.2M]</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Optimum Risk   95% CI [3.30–3.57]</t>
+          <t>Optimum Risk   95% CI [3.32–3.59]</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -1052,23 +1052,23 @@
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>€153,097,336</t>
+          <t>€152,962,125</t>
         </is>
       </c>
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>+0.31 pp</t>
+          <t>+0.34 pp</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>39.5%</t>
+          <t>39.6%</t>
         </is>
       </c>
       <c r="F6" s="10" t="n"/>
@@ -1080,12 +1080,12 @@
       <c r="H6" s="10" t="n"/>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>€+13,232,923</t>
+          <t>€+13,097,712</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+9.5%</t>
+          <t>+9.4%</t>
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr">
@@ -1137,7 +1137,7 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Recommended cutoffs change portfolio production +11.9% (€+12,624,715) at optimum risk 3.43% 95% CI [3.30–3.57].</t>
+          <t>Recommended cutoffs change portfolio production +11.8% (€+12,514,374) at optimum risk 3.45% 95% CI [3.32–3.59].</t>
         </is>
       </c>
     </row>
@@ -1229,22 +1229,22 @@
         <v>106306425.64</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>118931140.8007015</v>
+        <v>118820799.9413354</v>
       </c>
       <c r="D18" s="21" t="n">
-        <v>12624715.16070148</v>
+        <v>12514374.30133544</v>
       </c>
       <c r="E18" s="22" t="n">
-        <v>11.87577804887758</v>
+        <v>11.77198295022596</v>
       </c>
       <c r="F18" s="23" t="n">
         <v>3.648618</v>
       </c>
       <c r="G18" s="23" t="n">
-        <v>3.434567</v>
+        <v>3.451421</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>-0.214051</v>
+        <v>-0.1971970000000001</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -1257,22 +1257,22 @@
         <v>106306425.64</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>118931140.8007015</v>
+        <v>118820799.9413354</v>
       </c>
       <c r="D19" s="26" t="n">
-        <v>12624715.16070148</v>
+        <v>12514374.30133544</v>
       </c>
       <c r="E19" s="27" t="n">
-        <v>11.87577804887758</v>
+        <v>11.77198295022596</v>
       </c>
       <c r="F19" s="28" t="n">
         <v>3.648618</v>
       </c>
       <c r="G19" s="28" t="n">
-        <v>3.434567</v>
+        <v>3.451421</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>-0.214051</v>
+        <v>-0.1971970000000001</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -1285,22 +1285,22 @@
         <v>27401286.69</v>
       </c>
       <c r="C20" s="30" t="n">
-        <v>29672654.6219923</v>
+        <v>29620097.8776557</v>
       </c>
       <c r="D20" s="31" t="n">
-        <v>2271367.931992307</v>
+        <v>2218811.187655702</v>
       </c>
       <c r="E20" s="32" t="n">
-        <v>8.289274725267683</v>
+        <v>8.097470796747109</v>
       </c>
       <c r="F20" s="33" t="n">
         <v>2.132149</v>
       </c>
       <c r="G20" s="33" t="n">
-        <v>1.988801</v>
+        <v>1.98989</v>
       </c>
       <c r="H20" s="32" t="n">
-        <v>-0.143348</v>
+        <v>-0.1422590000000001</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -1313,22 +1313,22 @@
         <v>78905138.94999999</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>89258486.17870916</v>
+        <v>89200702.06367972</v>
       </c>
       <c r="D21" s="26" t="n">
-        <v>10353347.22870918</v>
+        <v>10295563.11367974</v>
       </c>
       <c r="E21" s="27" t="n">
-        <v>13.12125847122556</v>
+        <v>13.04802608636651</v>
       </c>
       <c r="F21" s="28" t="n">
         <v>4.169456</v>
       </c>
       <c r="G21" s="28" t="n">
-        <v>3.926883</v>
+        <v>3.948722</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>-0.2425730000000001</v>
+        <v>-0.2207340000000002</v>
       </c>
     </row>
     <row r="22"/>
@@ -1391,22 +1391,22 @@
         <v>139864412.8581818</v>
       </c>
       <c r="C25" s="20" t="n">
-        <v>153097336.1622182</v>
+        <v>152962124.8590652</v>
       </c>
       <c r="D25" s="21" t="n">
-        <v>13232923.30403641</v>
+        <v>13097712.00088337</v>
       </c>
       <c r="E25" s="22" t="n">
-        <v>9.461251102847859</v>
+        <v>9.364577974644662</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>3.510753</v>
+        <v>3.508981</v>
       </c>
       <c r="G25" s="23" t="n">
-        <v>3.822519</v>
+        <v>3.850114</v>
       </c>
       <c r="H25" s="34" t="n">
-        <v>0.311766</v>
+        <v>0.3411330000000001</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
@@ -1419,22 +1419,22 @@
         <v>139864412.8581818</v>
       </c>
       <c r="C26" s="30" t="n">
-        <v>153097336.1622182</v>
+        <v>152962124.8590652</v>
       </c>
       <c r="D26" s="31" t="n">
-        <v>13232923.30403641</v>
+        <v>13097712.00088337</v>
       </c>
       <c r="E26" s="32" t="n">
-        <v>9.461251102847859</v>
+        <v>9.364577974644662</v>
       </c>
       <c r="F26" s="33" t="n">
-        <v>3.510753</v>
+        <v>3.508981</v>
       </c>
       <c r="G26" s="33" t="n">
-        <v>3.822519</v>
+        <v>3.850114</v>
       </c>
       <c r="H26" s="35" t="n">
-        <v>0.311766</v>
+        <v>0.3411330000000001</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -1447,22 +1447,22 @@
         <v>34138254.80727272</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>35839138.75731456</v>
+        <v>35772222.75369629</v>
       </c>
       <c r="D27" s="26" t="n">
-        <v>1700883.950041838</v>
+        <v>1633967.946423568</v>
       </c>
       <c r="E27" s="27" t="n">
-        <v>4.982340074629374</v>
+        <v>4.786325357427092</v>
       </c>
       <c r="F27" s="28" t="n">
-        <v>2.049319</v>
+        <v>2.029839</v>
       </c>
       <c r="G27" s="28" t="n">
-        <v>1.988374</v>
+        <v>1.989857</v>
       </c>
       <c r="H27" s="27" t="n">
-        <v>-0.06094500000000003</v>
+        <v>-0.03998199999999996</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -1475,22 +1475,22 @@
         <v>105726158.0509091</v>
       </c>
       <c r="C28" s="30" t="n">
-        <v>117258197.4049037</v>
+        <v>117189902.1053689</v>
       </c>
       <c r="D28" s="31" t="n">
-        <v>11532039.35399458</v>
+        <v>11463744.05445981</v>
       </c>
       <c r="E28" s="32" t="n">
-        <v>10.90746090332885</v>
+        <v>10.84286449616358</v>
       </c>
       <c r="F28" s="33" t="n">
-        <v>3.951557</v>
+        <v>3.955353</v>
       </c>
       <c r="G28" s="33" t="n">
-        <v>4.357624</v>
+        <v>4.394509</v>
       </c>
       <c r="H28" s="35" t="n">
-        <v>0.4060670000000002</v>
+        <v>0.4391560000000001</v>
       </c>
     </row>
     <row r="29"/>
@@ -1593,34 +1593,34 @@
         <v>27401286.69</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>27519549.49543787</v>
-      </c>
-      <c r="F32" s="21" t="n">
-        <v>118262.805437874</v>
-      </c>
-      <c r="G32" s="22" t="n">
-        <v>0.4315958107216682</v>
+        <v>27396944.1838586</v>
+      </c>
+      <c r="F32" s="36" t="n">
+        <v>-4342.506141401827</v>
+      </c>
+      <c r="G32" s="34" t="n">
+        <v>-0.01584781835440819</v>
       </c>
       <c r="H32" s="23" t="n">
         <v>2.132149</v>
       </c>
       <c r="I32" s="23" t="n">
-        <v>1.499031</v>
+        <v>1.493039</v>
       </c>
       <c r="J32" s="22" t="n">
-        <v>-0.6331180000000001</v>
+        <v>-0.6391100000000001</v>
       </c>
       <c r="K32" s="23" t="n">
         <v>41.98258608500487</v>
       </c>
       <c r="L32" s="23" t="n">
-        <v>41.93466879695357</v>
+        <v>42.18659807574797</v>
       </c>
       <c r="M32" s="23" t="n">
         <v>40.83690506297156</v>
       </c>
       <c r="N32" s="23" t="n">
-        <v>40.95238445080282</v>
+        <v>41.21477788414601</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
@@ -1643,34 +1643,34 @@
         <v>106306425.64</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>118931140.8007015</v>
+        <v>118820799.9413354</v>
       </c>
       <c r="F33" s="21" t="n">
-        <v>12624715.16070148</v>
+        <v>12514374.30133544</v>
       </c>
       <c r="G33" s="22" t="n">
-        <v>11.87577804887758</v>
+        <v>11.77198295022596</v>
       </c>
       <c r="H33" s="23" t="n">
         <v>3.648618</v>
       </c>
       <c r="I33" s="23" t="n">
-        <v>3.434567</v>
+        <v>3.451421</v>
       </c>
       <c r="J33" s="22" t="n">
-        <v>-0.214051</v>
+        <v>-0.1971970000000001</v>
       </c>
       <c r="K33" s="23" t="n">
         <v>49.40800991602669</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>44.65004764647505</v>
+        <v>44.70670354196201</v>
       </c>
       <c r="M33" s="23" t="n">
         <v>47.19130464011302</v>
       </c>
       <c r="N33" s="23" t="n">
-        <v>42.52106566749935</v>
+        <v>42.57943365636294</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
@@ -1705,10 +1705,10 @@
         <v>2.132149</v>
       </c>
       <c r="I34" s="23" t="n">
-        <v>2.287386</v>
+        <v>2.293693</v>
       </c>
       <c r="J34" s="34" t="n">
-        <v>0.1552370000000001</v>
+        <v>0.1615440000000001</v>
       </c>
       <c r="K34" s="23" t="n">
         <v>41.98258608500487</v>
@@ -1743,34 +1743,34 @@
         <v>34138254.80727272</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>32686569.84439398</v>
+        <v>32542601.18044709</v>
       </c>
       <c r="F35" s="36" t="n">
-        <v>-1451684.962878749</v>
+        <v>-1595653.626825638</v>
       </c>
       <c r="G35" s="34" t="n">
-        <v>-4.25237016676519</v>
+        <v>-4.674092556382537</v>
       </c>
       <c r="H35" s="23" t="n">
-        <v>2.049319</v>
+        <v>2.029839</v>
       </c>
       <c r="I35" s="23" t="n">
-        <v>1.491246</v>
+        <v>1.490302</v>
       </c>
       <c r="J35" s="22" t="n">
-        <v>-0.558073</v>
+        <v>-0.5395369999999999</v>
       </c>
       <c r="K35" s="23" t="n">
         <v>33.80033360243112</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>36.1595678683062</v>
+        <v>36.49796714891394</v>
       </c>
       <c r="M35" s="23" t="n">
         <v>32.60829098689721</v>
       </c>
       <c r="N35" s="23" t="n">
-        <v>35.06993270255042</v>
+        <v>35.42540747170709</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
@@ -1793,34 +1793,34 @@
         <v>139864412.8581818</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>153097336.1622182</v>
+        <v>152962124.8590652</v>
       </c>
       <c r="F36" s="21" t="n">
-        <v>13232923.30403641</v>
+        <v>13097712.00088337</v>
       </c>
       <c r="G36" s="22" t="n">
-        <v>9.461251102847859</v>
+        <v>9.364577974644662</v>
       </c>
       <c r="H36" s="23" t="n">
-        <v>3.510753</v>
+        <v>3.508981</v>
       </c>
       <c r="I36" s="23" t="n">
-        <v>3.822519</v>
+        <v>3.850114</v>
       </c>
       <c r="J36" s="34" t="n">
-        <v>0.311766</v>
+        <v>0.3411330000000001</v>
       </c>
       <c r="K36" s="23" t="n">
         <v>44.00757330718467</v>
       </c>
       <c r="L36" s="23" t="n">
-        <v>39.52137673041613</v>
+        <v>39.55939616633726</v>
       </c>
       <c r="M36" s="23" t="n">
         <v>41.6561394100917</v>
       </c>
       <c r="N36" s="23" t="n">
-        <v>37.16207316209882</v>
+        <v>37.20009259801994</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
@@ -1852,13 +1852,13 @@
         <v>5.989891454447482</v>
       </c>
       <c r="H37" s="23" t="n">
-        <v>2.049319</v>
+        <v>2.029839</v>
       </c>
       <c r="I37" s="23" t="n">
-        <v>2.287231</v>
+        <v>2.293668</v>
       </c>
       <c r="J37" s="34" t="n">
-        <v>0.2379119999999997</v>
+        <v>0.2638289999999999</v>
       </c>
       <c r="K37" s="23" t="n">
         <v>33.80033360243112</v>
@@ -1930,25 +1930,25 @@
         </is>
       </c>
       <c r="B41" s="25" t="n">
-        <v>89258486.17870916</v>
+        <v>89200702.06367972</v>
       </c>
       <c r="C41" s="26" t="n">
-        <v>10353347.22870918</v>
+        <v>10295563.11367974</v>
       </c>
       <c r="D41" s="27" t="n">
-        <v>13.12125847122556</v>
+        <v>13.04802608636651</v>
       </c>
       <c r="E41" s="28" t="n">
-        <v>3.926883</v>
+        <v>3.948722</v>
       </c>
       <c r="F41" s="27" t="n">
-        <v>-0.2425730000000001</v>
+        <v>-0.2207340000000002</v>
       </c>
       <c r="G41" s="28" t="n">
-        <v>45.71876067166517</v>
+        <v>45.76940007117907</v>
       </c>
       <c r="H41" s="28" t="n">
-        <v>43.43715845519815</v>
+        <v>43.48832402882581</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
@@ -1958,25 +1958,25 @@
         </is>
       </c>
       <c r="B42" s="30" t="n">
-        <v>29672654.6219923</v>
+        <v>29620097.8776557</v>
       </c>
       <c r="C42" s="31" t="n">
-        <v>2271367.931992307</v>
+        <v>2218811.187655702</v>
       </c>
       <c r="D42" s="32" t="n">
-        <v>8.289274725267683</v>
+        <v>8.097470796747109</v>
       </c>
       <c r="E42" s="33" t="n">
-        <v>1.988801</v>
+        <v>1.98989</v>
       </c>
       <c r="F42" s="32" t="n">
-        <v>-0.143348</v>
+        <v>-0.1422590000000001</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>37.66285234135594</v>
+        <v>37.75884380347808</v>
       </c>
       <c r="H42" s="33" t="n">
-        <v>36.53169426994965</v>
+        <v>36.63715130960228</v>
       </c>
     </row>
     <row r="43"/>
@@ -2036,25 +2036,25 @@
         </is>
       </c>
       <c r="B46" s="30" t="n">
-        <v>117258197.4049037</v>
+        <v>117189902.1053689</v>
       </c>
       <c r="C46" s="31" t="n">
-        <v>11532039.35399458</v>
+        <v>11463744.05445981</v>
       </c>
       <c r="D46" s="32" t="n">
-        <v>10.90746090332885</v>
+        <v>10.84286449616358</v>
       </c>
       <c r="E46" s="33" t="n">
-        <v>4.357624</v>
+        <v>4.394509</v>
       </c>
       <c r="F46" s="35" t="n">
-        <v>0.4060670000000002</v>
+        <v>0.4391560000000001</v>
       </c>
       <c r="G46" s="33" t="n">
-        <v>40.7300486534887</v>
+        <v>40.75824671913305</v>
       </c>
       <c r="H46" s="33" t="n">
-        <v>38.20430792631301</v>
+        <v>38.23250599195735</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
@@ -2064,25 +2064,25 @@
         </is>
       </c>
       <c r="B47" s="25" t="n">
-        <v>35839138.75731456</v>
+        <v>35772222.75369629</v>
       </c>
       <c r="C47" s="26" t="n">
-        <v>1700883.950041838</v>
+        <v>1633967.946423568</v>
       </c>
       <c r="D47" s="27" t="n">
-        <v>4.982340074629374</v>
+        <v>4.786325357427092</v>
       </c>
       <c r="E47" s="28" t="n">
-        <v>1.988374</v>
+        <v>1.989857</v>
       </c>
       <c r="F47" s="27" t="n">
-        <v>-0.06094500000000003</v>
+        <v>-0.03998199999999996</v>
       </c>
       <c r="G47" s="28" t="n">
-        <v>31.02871271964337</v>
+        <v>31.13574145105142</v>
       </c>
       <c r="H47" s="28" t="n">
-        <v>29.83887031122347</v>
+        <v>29.94589904263152</v>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1">
@@ -2693,14 +2693,14 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C56" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D56" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="E56" s="41" t="inlineStr">
@@ -2798,9 +2798,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C57" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="D57" s="41" t="inlineStr">
@@ -3108,9 +3108,9 @@
       <c r="A60" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="B60" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B60" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="C60" s="41" t="inlineStr">
@@ -3209,180 +3209,286 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="42" t="inlineStr">
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="B61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U61" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="26" customHeight="1">
+      <c r="A62" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U62" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  A  Accept  </t>
         </is>
       </c>
-      <c r="B62" s="43" t="inlineStr">
+      <c r="B64" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  R  Reject  </t>
         </is>
       </c>
-      <c r="C62" s="44" t="inlineStr">
+      <c r="C64" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  —  N/A  </t>
         </is>
       </c>
     </row>
-    <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="37" t="inlineStr">
+    <row r="66" ht="28" customHeight="1">
+      <c r="A66" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  new  |  Base</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="38" t="inlineStr">
+    <row r="67" ht="26" customHeight="1">
+      <c r="A67" s="38" t="inlineStr">
         <is>
           <t>new_efx_clus \ sc_octroi_new_clus</t>
         </is>
       </c>
-      <c r="B65" s="39" t="n">
+      <c r="B67" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="C65" s="39" t="n">
+      <c r="C67" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="D65" s="39" t="n">
+      <c r="D67" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="E65" s="39" t="n">
+      <c r="E67" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="F65" s="39" t="n">
+      <c r="F67" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="G65" s="39" t="n">
+      <c r="G67" s="39" t="n">
         <v>6</v>
       </c>
-      <c r="H65" s="39" t="n">
+      <c r="H67" s="39" t="n">
         <v>7</v>
       </c>
-      <c r="I65" s="39" t="n">
+      <c r="I67" s="39" t="n">
         <v>8</v>
       </c>
-      <c r="J65" s="39" t="n">
+      <c r="J67" s="39" t="n">
         <v>9</v>
       </c>
-      <c r="K65" s="39" t="n">
+      <c r="K67" s="39" t="n">
         <v>10</v>
       </c>
-    </row>
-    <row r="66" ht="26" customHeight="1">
-      <c r="A66" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="B66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="I66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J66" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="K66" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="26" customHeight="1">
-      <c r="A67" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="B67" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C67" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D67" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E67" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F67" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G67" s="40" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H67" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I67" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J67" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K67" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="L67" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="M67" s="39" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="68" ht="26" customHeight="1">
       <c r="A68" s="39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B68" s="40" t="inlineStr">
         <is>
@@ -3414,22 +3520,32 @@
           <t>R</t>
         </is>
       </c>
-      <c r="H68" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I68" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J68" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K68" s="41" t="inlineStr">
+      <c r="H68" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I68" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J68" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="K68" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="L68" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M68" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3437,7 +3553,7 @@
     </row>
     <row r="69" ht="26" customHeight="1">
       <c r="A69" s="39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B69" s="40" t="inlineStr">
         <is>
@@ -3459,19 +3575,19 @@
           <t>R</t>
         </is>
       </c>
-      <c r="F69" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G69" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H69" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F69" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G69" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H69" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="I69" s="41" t="inlineStr">
@@ -3485,6 +3601,16 @@
         </is>
       </c>
       <c r="K69" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L69" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M69" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3492,41 +3618,41 @@
     </row>
     <row r="70" ht="26" customHeight="1">
       <c r="A70" s="39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B70" s="40" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C70" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D70" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E70" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F70" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G70" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H70" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D70" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E70" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F70" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G70" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H70" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="I70" s="41" t="inlineStr">
@@ -3540,6 +3666,16 @@
         </is>
       </c>
       <c r="K70" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L70" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M70" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3547,26 +3683,26 @@
     </row>
     <row r="71" ht="26" customHeight="1">
       <c r="A71" s="39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B71" s="40" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C71" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D71" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E71" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C71" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D71" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E71" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="F71" s="41" t="inlineStr">
@@ -3595,6 +3731,16 @@
         </is>
       </c>
       <c r="K71" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L71" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M71" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3602,11 +3748,11 @@
     </row>
     <row r="72" ht="26" customHeight="1">
       <c r="A72" s="39" t="n">
-        <v>7</v>
-      </c>
-      <c r="B72" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>5</v>
+      </c>
+      <c r="B72" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="C72" s="41" t="inlineStr">
@@ -3650,6 +3796,16 @@
         </is>
       </c>
       <c r="K72" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L72" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M72" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3657,11 +3813,11 @@
     </row>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="39" t="n">
-        <v>8</v>
-      </c>
-      <c r="B73" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>6</v>
+      </c>
+      <c r="B73" s="40" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="C73" s="41" t="inlineStr">
@@ -3705,6 +3861,16 @@
         </is>
       </c>
       <c r="K73" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L73" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M73" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3712,7 +3878,7 @@
     </row>
     <row r="74" ht="26" customHeight="1">
       <c r="A74" s="39" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B74" s="41" t="inlineStr">
         <is>
@@ -3760,6 +3926,16 @@
         </is>
       </c>
       <c r="K74" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L74" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M74" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3767,7 +3943,7 @@
     </row>
     <row r="75" ht="26" customHeight="1">
       <c r="A75" s="39" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B75" s="41" t="inlineStr">
         <is>
@@ -3815,6 +3991,16 @@
         </is>
       </c>
       <c r="K75" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L75" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M75" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3822,7 +4008,7 @@
     </row>
     <row r="76" ht="26" customHeight="1">
       <c r="A76" s="39" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B76" s="41" t="inlineStr">
         <is>
@@ -3870,6 +4056,16 @@
         </is>
       </c>
       <c r="K76" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L76" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M76" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3877,7 +4073,7 @@
     </row>
     <row r="77" ht="26" customHeight="1">
       <c r="A77" s="39" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B77" s="41" t="inlineStr">
         <is>
@@ -3925,6 +4121,16 @@
         </is>
       </c>
       <c r="K77" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L77" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M77" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3932,7 +4138,7 @@
     </row>
     <row r="78" ht="26" customHeight="1">
       <c r="A78" s="39" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B78" s="41" t="inlineStr">
         <is>
@@ -3980,6 +4186,16 @@
         </is>
       </c>
       <c r="K78" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L78" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M78" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3987,7 +4203,7 @@
     </row>
     <row r="79" ht="26" customHeight="1">
       <c r="A79" s="39" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B79" s="41" t="inlineStr">
         <is>
@@ -4035,6 +4251,16 @@
         </is>
       </c>
       <c r="K79" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L79" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M79" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4042,7 +4268,7 @@
     </row>
     <row r="80" ht="26" customHeight="1">
       <c r="A80" s="39" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B80" s="41" t="inlineStr">
         <is>
@@ -4090,6 +4316,16 @@
         </is>
       </c>
       <c r="K80" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L80" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M80" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4097,7 +4333,7 @@
     </row>
     <row r="81" ht="26" customHeight="1">
       <c r="A81" s="39" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B81" s="41" t="inlineStr">
         <is>
@@ -4145,6 +4381,16 @@
         </is>
       </c>
       <c r="K81" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L81" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M81" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4152,7 +4398,7 @@
     </row>
     <row r="82" ht="26" customHeight="1">
       <c r="A82" s="39" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B82" s="41" t="inlineStr">
         <is>
@@ -4200,6 +4446,16 @@
         </is>
       </c>
       <c r="K82" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L82" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M82" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4207,7 +4463,7 @@
     </row>
     <row r="83" ht="26" customHeight="1">
       <c r="A83" s="39" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B83" s="41" t="inlineStr">
         <is>
@@ -4255,6 +4511,16 @@
         </is>
       </c>
       <c r="K83" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L83" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M83" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4262,7 +4528,7 @@
     </row>
     <row r="84" ht="26" customHeight="1">
       <c r="A84" s="39" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B84" s="41" t="inlineStr">
         <is>
@@ -4310,6 +4576,16 @@
         </is>
       </c>
       <c r="K84" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L84" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M84" s="41" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4317,71 +4593,211 @@
     </row>
     <row r="85" ht="26" customHeight="1">
       <c r="A85" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="B85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M85" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M86" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="B85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K85" s="41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="42" t="inlineStr">
+      <c r="B87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M87" s="41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  A  Accept  </t>
         </is>
       </c>
-      <c r="B87" s="43" t="inlineStr">
+      <c r="B89" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  R  Reject  </t>
         </is>
       </c>
-      <c r="C87" s="44" t="inlineStr">
+      <c r="C89" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  —  N/A  </t>
         </is>
@@ -4390,7 +4806,6 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A64:L64"/>
     <mergeCell ref="A10:L10"/>
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="A11:L11"/>
@@ -4399,6 +4814,7 @@
     <mergeCell ref="A30:N30"/>
     <mergeCell ref="A13:L13"/>
     <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A66:L66"/>
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A9:L9"/>
     <mergeCell ref="A2:J2"/>
@@ -4503,7 +4919,7 @@
       </c>
       <c r="B9" s="48" t="inlineStr">
         <is>
-          <t>20260617T085641Z_b53c771578b7  ·  git b53c771578b7 (dirty)  ·  cfg ac4ea54f85d7</t>
+          <t>20260617T114353Z_b1bd4685bfc4  ·  git b1bd4685bfc4 (dirty)  ·  cfg e3588add6f53</t>
         </is>
       </c>
     </row>
@@ -5038,14 +5454,14 @@
         <v>219</v>
       </c>
       <c r="D7" t="n">
-        <v>1.9888</v>
+        <v>1.9899</v>
       </c>
       <c r="E7" t="n">
-        <v>1.8467</v>
+        <v>1.846</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[1.6338, 2.0628]</t>
+          <t>[1.6405, 2.0601]</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -5057,10 +5473,10 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>0.9558</v>
+        <v>0.9519</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9696</v>
+        <v>0.9667</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -5091,14 +5507,14 @@
         <v>1023</v>
       </c>
       <c r="D8" t="n">
-        <v>3.9269</v>
+        <v>3.9487</v>
       </c>
       <c r="E8" t="n">
-        <v>3.5636</v>
+        <v>3.5738</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[3.3809, 3.7514]</t>
+          <t>[3.3926, 3.7655]</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -5110,10 +5526,10 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>0.8649</v>
+        <v>0.8645</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8947000000000001</v>
+        <v>0.8943</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -5158,13 +5574,13 @@
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
     <col width="23" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
@@ -5377,13 +5793,13 @@
         </is>
       </c>
       <c r="B6" s="33" t="n">
-        <v>5.054906</v>
+        <v>5.150228</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>2535473.32199231</v>
+        <v>2504925.557655705</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.09253117748363331</v>
+        <v>0.0914163479253647</v>
       </c>
       <c r="E6" s="33" t="inlineStr"/>
       <c r="F6" s="33" t="inlineStr"/>
@@ -5424,13 +5840,13 @@
         </is>
       </c>
       <c r="B7" s="28" t="n">
-        <v>30.014318</v>
+        <v>28.081723</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>264105.39</v>
+        <v>286114.37</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0.0096384302309564</v>
+        <v>0.0104416399578935</v>
       </c>
       <c r="E7" s="28" t="inlineStr"/>
       <c r="F7" s="28" t="inlineStr"/>
@@ -5459,31 +5875,31 @@
         </is>
       </c>
       <c r="B8" s="59" t="n">
-        <v>1.988801</v>
+        <v>1.98989</v>
       </c>
       <c r="C8" s="60" t="n">
-        <v>29672654.6219923</v>
+        <v>29620097.8776557</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>1.082892747252677</v>
+        <v>1.080974707967471</v>
       </c>
       <c r="E8" s="59" t="n">
-        <v>37.66285234135594</v>
+        <v>37.75884380347808</v>
       </c>
       <c r="F8" s="59" t="n">
-        <v>36.53169426994965</v>
+        <v>36.63715130960228</v>
       </c>
       <c r="G8" s="60" t="n">
-        <v>29420298.83583964</v>
+        <v>29376868.52095652</v>
       </c>
       <c r="H8" s="60" t="n">
-        <v>29798968.14113409</v>
+        <v>29758992.84995979</v>
       </c>
       <c r="I8" s="59" t="n">
-        <v>1.784585</v>
+        <v>1.7857375</v>
       </c>
       <c r="J8" s="59" t="n">
-        <v>2.1893175</v>
+        <v>2.1893125</v>
       </c>
       <c r="K8" s="61" t="inlineStr">
         <is>
@@ -5491,22 +5907,22 @@
         </is>
       </c>
       <c r="L8" s="61" t="n">
-        <v>1.632395</v>
+        <v>1.6311975</v>
       </c>
       <c r="M8" s="61" t="n">
-        <v>2.0572225</v>
+        <v>2.0560125</v>
       </c>
       <c r="N8" s="61" t="n">
-        <v>1.959694888736929</v>
+        <v>1.960090531079756</v>
       </c>
       <c r="O8" s="61" t="n">
-        <v>1.999536113368798</v>
+        <v>1.999583554870518</v>
       </c>
       <c r="P8" s="61" t="n">
-        <v>0.0054338183276409</v>
+        <v>0.0062414739612841</v>
       </c>
       <c r="Q8" s="61" t="n">
-        <v>92.8</v>
+        <v>93.2</v>
       </c>
       <c r="R8" s="61" t="inlineStr"/>
       <c r="S8" s="61" t="inlineStr"/>
@@ -5522,13 +5938,13 @@
         </is>
       </c>
       <c r="B9" s="63" t="n">
-        <v>-0.1411989999999998</v>
+        <v>-0.1401099999999999</v>
       </c>
       <c r="C9" s="64" t="n">
-        <v>2271367.931992307</v>
+        <v>2218811.187655702</v>
       </c>
       <c r="D9" s="63" t="n">
-        <v>0.0828927472526768</v>
+        <v>0.080974707967471</v>
       </c>
       <c r="E9" s="63" t="inlineStr"/>
       <c r="F9" s="63" t="inlineStr"/>
@@ -5647,7 +6063,7 @@
         </is>
       </c>
       <c r="B5" s="28" t="n">
-        <v>2.049319</v>
+        <v>2.029839</v>
       </c>
       <c r="C5" s="25" t="n">
         <v>34138254.80727272</v>
@@ -5672,13 +6088,13 @@
         </is>
       </c>
       <c r="B6" s="33" t="n">
-        <v>7.605546</v>
+        <v>8.190300000000001</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>1721132.128223661</v>
+        <v>1657203.04460539</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.0504165235727573</v>
+        <v>0.0485438712072751</v>
       </c>
       <c r="E6" s="33" t="inlineStr"/>
       <c r="F6" s="33" t="inlineStr"/>
@@ -5691,18 +6107,18 @@
         </is>
       </c>
       <c r="B7" s="28" t="n">
-        <v>17.112499</v>
+        <v>17.429285</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>20248.17818181818</v>
+        <v>23235.09818181818</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0.0005931228264634</v>
+        <v>0.0006806176330041</v>
       </c>
       <c r="E7" s="28" t="inlineStr"/>
       <c r="F7" s="28" t="inlineStr"/>
       <c r="G7" s="28" t="n">
-        <v>11.799538</v>
+        <v>10.995671</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -5712,22 +6128,22 @@
         </is>
       </c>
       <c r="B8" s="59" t="n">
-        <v>1.988374</v>
+        <v>1.989857</v>
       </c>
       <c r="C8" s="60" t="n">
-        <v>35839138.75731456</v>
+        <v>35772222.75369629</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>1.049823400746294</v>
+        <v>1.047863253574271</v>
       </c>
       <c r="E8" s="59" t="n">
-        <v>31.02871271964337</v>
+        <v>31.13574145105142</v>
       </c>
       <c r="F8" s="59" t="n">
-        <v>29.83887031122347</v>
+        <v>29.94589904263152</v>
       </c>
       <c r="G8" s="59" t="n">
-        <v>0.955581</v>
+        <v>0.962422</v>
       </c>
     </row>
   </sheetData>
@@ -5768,9 +6184,9 @@
     <col width="20" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
@@ -5978,13 +6394,13 @@
         </is>
       </c>
       <c r="B6" s="33" t="n">
-        <v>9.108454</v>
+        <v>9.367380000000001</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>12117832.86870918</v>
+        <v>12057440.25367973</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.1535746977948789</v>
+        <v>0.1528093152629792</v>
       </c>
       <c r="E6" s="33" t="inlineStr"/>
       <c r="F6" s="33" t="inlineStr"/>
@@ -6000,13 +6416,13 @@
       <c r="P6" s="57" t="inlineStr"/>
       <c r="Q6" s="57" t="inlineStr"/>
       <c r="R6" s="57" t="n">
-        <v>1.019409436786817</v>
+        <v>1.016317662406026</v>
       </c>
       <c r="S6" s="57" t="n">
-        <v>1.635512048454683</v>
+        <v>1.629848654227153</v>
       </c>
       <c r="T6" s="57" t="n">
-        <v>2.189999279030957</v>
+        <v>2.180010919745711</v>
       </c>
       <c r="U6" s="57" t="n">
         <v>1</v>
@@ -6025,13 +6441,13 @@
         </is>
       </c>
       <c r="B7" s="28" t="n">
-        <v>29.040945</v>
+        <v>28.69377</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>1764485.64</v>
+        <v>1761877.14</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0.0223621130826232</v>
+        <v>0.0223290543993142</v>
       </c>
       <c r="E7" s="28" t="inlineStr"/>
       <c r="F7" s="28" t="inlineStr"/>
@@ -6060,31 +6476,31 @@
         </is>
       </c>
       <c r="B8" s="59" t="n">
-        <v>3.926883</v>
+        <v>3.948722</v>
       </c>
       <c r="C8" s="60" t="n">
-        <v>89258486.17870916</v>
+        <v>89200702.06367972</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>1.131212584712256</v>
+        <v>1.130480260863665</v>
       </c>
       <c r="E8" s="59" t="n">
-        <v>45.71876067166517</v>
+        <v>45.76940007117907</v>
       </c>
       <c r="F8" s="59" t="n">
-        <v>43.43715845519815</v>
+        <v>43.48832402882581</v>
       </c>
       <c r="G8" s="60" t="n">
-        <v>87608510.83146046</v>
+        <v>87585864.46647418</v>
       </c>
       <c r="H8" s="60" t="n">
-        <v>88180086.83031934</v>
+        <v>88147152.98152852</v>
       </c>
       <c r="I8" s="59" t="n">
-        <v>3.7612875</v>
+        <v>3.7820725</v>
       </c>
       <c r="J8" s="59" t="n">
-        <v>4.098610000000001</v>
+        <v>4.118945</v>
       </c>
       <c r="K8" s="61" t="inlineStr">
         <is>
@@ -6092,19 +6508,19 @@
         </is>
       </c>
       <c r="L8" s="61" t="n">
-        <v>3.387555</v>
+        <v>3.399155</v>
       </c>
       <c r="M8" s="61" t="n">
-        <v>3.74546</v>
+        <v>3.7585025</v>
       </c>
       <c r="N8" s="61" t="n">
-        <v>3.758423415294931</v>
+        <v>3.774041379224162</v>
       </c>
       <c r="O8" s="61" t="n">
-        <v>4.106559417431397</v>
+        <v>4.13013995735678</v>
       </c>
       <c r="P8" s="61" t="n">
-        <v>-0.0009056646292686</v>
+        <v>-0.000550433036892</v>
       </c>
       <c r="Q8" s="61" t="n">
         <v>0</v>
@@ -6123,13 +6539,13 @@
         </is>
       </c>
       <c r="B9" s="63" t="n">
-        <v>-0.2431169999999998</v>
+        <v>-0.2212779999999998</v>
       </c>
       <c r="C9" s="64" t="n">
-        <v>10353347.22870918</v>
+        <v>10295563.11367974</v>
       </c>
       <c r="D9" s="63" t="n">
-        <v>0.1312125847122556</v>
+        <v>0.130480260863665</v>
       </c>
       <c r="E9" s="63" t="inlineStr"/>
       <c r="F9" s="63" t="inlineStr"/>
@@ -6248,7 +6664,7 @@
         </is>
       </c>
       <c r="B5" s="28" t="n">
-        <v>3.951557</v>
+        <v>3.955353</v>
       </c>
       <c r="C5" s="25" t="n">
         <v>105726158.0509091</v>
@@ -6273,13 +6689,13 @@
         </is>
       </c>
       <c r="B6" s="33" t="n">
-        <v>14.057634</v>
+        <v>14.933609</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>11532039.35399458</v>
+        <v>11463744.0544598</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.1090746090332885</v>
+        <v>0.1084286449616357</v>
       </c>
       <c r="E6" s="33" t="inlineStr"/>
       <c r="F6" s="33" t="inlineStr"/>
@@ -6309,19 +6725,19 @@
         </is>
       </c>
       <c r="B8" s="59" t="n">
-        <v>4.357624</v>
+        <v>4.394509</v>
       </c>
       <c r="C8" s="60" t="n">
-        <v>117258197.4049036</v>
+        <v>117189902.1053689</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>1.109074609033289</v>
+        <v>1.108428644961636</v>
       </c>
       <c r="E8" s="59" t="n">
-        <v>40.7300486534887</v>
+        <v>40.75824671913305</v>
       </c>
       <c r="F8" s="59" t="n">
-        <v>38.20430792631301</v>
+        <v>38.23250599195735</v>
       </c>
       <c r="G8" s="59" t="n">
         <v>2.527868</v>

</xml_diff>

<commit_message>
reports: refresh consolidated reports (MR production reconcile fix)
Regenerated after the MR audit/production fix; MR-period production now
reflects the re-optimized mask consistent with the reported MR risk.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -961,7 +961,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 17 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260617T151044Z_6b811ac36044  |  git 6b811ac36044 (dirty)  |  data sha 5f0d5d9c42a4</t>
+          <t xml:space="preserve">  Generated 18 Jun 2026  |  2 segment(s)  |  Consolidated portfolio view  |  run 20260618T172607Z_14e863e5c5b6  |  git 14e863e5c5b6 (dirty)  |  data sha 5f0d5d9c42a4</t>
         </is>
       </c>
     </row>
@@ -7612,7 +7612,7 @@
       </c>
       <c r="B9" s="48" t="inlineStr">
         <is>
-          <t>20260617T151044Z_6b811ac36044  ·  git 6b811ac36044 (dirty)  ·  cfg e3588add6f53</t>
+          <t>20260618T172607Z_14e863e5c5b6  ·  git 14e863e5c5b6 (dirty)  ·  cfg e3588add6f53</t>
         </is>
       </c>
     </row>
@@ -8784,10 +8784,10 @@
         <v>8.190300000000001</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>1657203.04460539</v>
+        <v>1356727.487732399</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.0485438712072751</v>
+        <v>0.039742145443339</v>
       </c>
       <c r="E6" s="33" t="inlineStr"/>
       <c r="F6" s="33" t="inlineStr"/>
@@ -8803,10 +8803,10 @@
         <v>17.429285</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>23235.09818181818</v>
+        <v>462247.2654545454</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0.0006806176330041</v>
+        <v>0.0135404480417689</v>
       </c>
       <c r="E7" s="28" t="inlineStr"/>
       <c r="F7" s="28" t="inlineStr"/>
@@ -8824,16 +8824,16 @@
         <v>1.989857</v>
       </c>
       <c r="C8" s="60" t="n">
-        <v>35772222.75369629</v>
+        <v>35032735.02955058</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>1.047863253574271</v>
+        <v>1.02620169740157</v>
       </c>
       <c r="E8" s="59" t="n">
-        <v>31.13574145105142</v>
+        <v>32.27747064584081</v>
       </c>
       <c r="F8" s="59" t="n">
-        <v>29.94589904263152</v>
+        <v>31.10856858438135</v>
       </c>
       <c r="G8" s="59" t="n">
         <v>0.962422</v>
@@ -9385,10 +9385,10 @@
         <v>13.203591</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>12015934.30998714</v>
+        <v>7233672.72181139</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.1136514797426124</v>
+        <v>0.0684189500041063</v>
       </c>
       <c r="E6" s="33" t="inlineStr"/>
       <c r="F6" s="33" t="inlineStr"/>
@@ -9404,10 +9404,10 @@
         <v>14.961573</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>0</v>
+        <v>2227777.32</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0</v>
+        <v>0.0210712028231205</v>
       </c>
       <c r="E7" s="28" t="inlineStr"/>
       <c r="F7" s="28" t="inlineStr"/>
@@ -9425,16 +9425,16 @@
         <v>3.991845</v>
       </c>
       <c r="C8" s="60" t="n">
-        <v>117742092.3608962</v>
+        <v>110732053.4527205</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>1.113651479742612</v>
+        <v>1.047347747180986</v>
       </c>
       <c r="E8" s="59" t="n">
-        <v>40.53228487479426</v>
+        <v>43.82693712018779</v>
       </c>
       <c r="F8" s="59" t="n">
-        <v>38.00676484193427</v>
+        <v>41.41714674447889</v>
       </c>
       <c r="G8" s="59" t="n">
         <v>2.406012</v>

</xml_diff>

<commit_message>
chore(output): regenerated consolidated reports with all audit fixes (F1-F11)
Full batch on main at 73da737: all eleven audit findings applied,
including the F8 usable-risk gate (with the vacuous phantom-floor-cell
refinement — ab's 4 empty floor cells dropped with a warning instead of
failing the segment). TOTAL main/base: Risk 1.71%->1.17%, HRI
1.74%->1.17%, production EUR 290.6M — full 6-segment coverage restored.
direct-pl-new still fails its pre-existing DQ booked-ratio gate (0.8% <
1%, predates the audit work; artifacts stale from Sep 7, tracked
separately).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015LhKMLGSYEFjhy3snTVrNE
</commit_message>
<xml_diff>
--- a/output/consolidated_risk_production.xlsx
+++ b/output/consolidated_risk_production.xlsx
@@ -4454,7 +4454,7 @@
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="29" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
@@ -4473,7 +4473,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 08 Sep 2026  |  6 segment(s)  |  Consolidated portfolio view  |  run 20260908T080239Z_8554dd50756a  |  git 8554dd50756a (dirty)  |  data sha 4b5c3f489dcc</t>
+          <t xml:space="preserve">  Generated 08 Sep 2026  |  6 segment(s)  |  Consolidated portfolio view  |  run 20260908T125042Z_73da737810a7  |  git 73da737810a7 (dirty)  |  data sha 4b5c3f489dcc</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>€290,638,590</t>
+          <t>€290,631,739</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
@@ -4520,7 +4520,7 @@
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>€-28,799,382</t>
+          <t>€-28,806,233</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -4537,7 +4537,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Optimum Production   95% CI [€287.6M–€293.6M]</t>
+          <t>Optimum Production   95% CI [€287.6M–€293.7M]</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -4569,13 +4569,13 @@
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>€330,169,136</t>
+          <t>€329,740,211</t>
         </is>
       </c>
       <c r="B6" s="11" t="n"/>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>1.20%</t>
+          <t>1.19%</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -4585,24 +4585,24 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>65.8%</t>
+          <t>65.7%</t>
         </is>
       </c>
       <c r="F6" s="11" t="n"/>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>64.9%</t>
         </is>
       </c>
       <c r="H6" s="11" t="n"/>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>€-18,034,732</t>
+          <t>€-18,463,656</t>
         </is>
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>-5.2%</t>
+          <t>-5.3%</t>
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr">
@@ -4652,7 +4652,7 @@
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1.18%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -4726,7 +4726,7 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Recommended cutoffs change portfolio production -9.0% (€-28,799,382) at optimum risk 1.17% 95% CI [1.01–1.33].</t>
+          <t>Recommended cutoffs change portfolio production -9.0% (€-28,806,233) at optimum risk 1.17% 95% CI [1.01–1.33].</t>
         </is>
       </c>
     </row>
@@ -4828,28 +4828,28 @@
         <v>319437971.72</v>
       </c>
       <c r="C21" s="21" t="n">
-        <v>290638589.9751463</v>
+        <v>290631738.6745474</v>
       </c>
       <c r="D21" s="22" t="n">
-        <v>-28799381.74485373</v>
+        <v>-28806233.04545259</v>
       </c>
       <c r="E21" s="23" t="n">
-        <v>-9.015641312078429</v>
+        <v>-9.017786110507361</v>
       </c>
       <c r="F21" s="24" t="n">
         <v>1.709876</v>
       </c>
       <c r="G21" s="24" t="n">
-        <v>1.16794</v>
+        <v>1.167463</v>
       </c>
       <c r="H21" s="25" t="n">
-        <v>-0.541936</v>
+        <v>-0.542413</v>
       </c>
       <c r="I21" s="24" t="n">
         <v>1.734517</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>1.17538</v>
+        <v>1.173858</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -4874,10 +4874,10 @@
         <v>1.307143</v>
       </c>
       <c r="G22" s="30" t="n">
-        <v>0.6919</v>
+        <v>0.691937</v>
       </c>
       <c r="H22" s="31" t="n">
-        <v>-0.615243</v>
+        <v>-0.6152059999999999</v>
       </c>
       <c r="I22" s="30" t="n">
         <v>1.312484</v>
@@ -4896,22 +4896,22 @@
         <v>147407667.46</v>
       </c>
       <c r="C23" s="33" t="n">
-        <v>128874581.9178167</v>
+        <v>128880087.3089723</v>
       </c>
       <c r="D23" s="34" t="n">
-        <v>-18533085.54218332</v>
+        <v>-18527580.15102771</v>
       </c>
       <c r="E23" s="35" t="n">
-        <v>-12.57267404167588</v>
+        <v>-12.56893923516922</v>
       </c>
       <c r="F23" s="36" t="n">
         <v>1.95724</v>
       </c>
       <c r="G23" s="36" t="n">
-        <v>1.256799</v>
+        <v>1.256906</v>
       </c>
       <c r="H23" s="37" t="n">
-        <v>-0.7004410000000001</v>
+        <v>-0.700334</v>
       </c>
       <c r="I23" s="36" t="n">
         <v>1.941038</v>
@@ -4930,28 +4930,28 @@
         <v>96048368.26000001</v>
       </c>
       <c r="C24" s="27" t="n">
-        <v>93416888.58999512</v>
+        <v>93404531.89824064</v>
       </c>
       <c r="D24" s="28" t="n">
-        <v>-2631479.670004889</v>
+        <v>-2643836.361759365</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>-2.739744274344728</v>
+        <v>-2.752609346368676</v>
       </c>
       <c r="F24" s="30" t="n">
         <v>1.649876</v>
       </c>
       <c r="G24" s="30" t="n">
-        <v>1.393761</v>
+        <v>1.39217</v>
       </c>
       <c r="H24" s="31" t="n">
-        <v>-0.2561149999999999</v>
+        <v>-0.257706</v>
       </c>
       <c r="I24" s="30" t="n">
         <v>1.750748</v>
       </c>
       <c r="J24" s="30" t="n">
-        <v>1.459124</v>
+        <v>1.454767</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -4976,10 +4976,10 @@
         <v>2.06382</v>
       </c>
       <c r="G25" s="36" t="n">
-        <v>0.788784</v>
+        <v>0.788872</v>
       </c>
       <c r="H25" s="37" t="n">
-        <v>-1.275036</v>
+        <v>-1.274948</v>
       </c>
       <c r="I25" s="36" t="n">
         <v>1.914059</v>
@@ -5044,10 +5044,10 @@
         <v>1.642293</v>
       </c>
       <c r="G27" s="36" t="n">
-        <v>1.132772</v>
+        <v>1.132763</v>
       </c>
       <c r="H27" s="37" t="n">
-        <v>-0.5095210000000001</v>
+        <v>-0.50953</v>
       </c>
       <c r="I27" s="36" t="n">
         <v>1.667502</v>
@@ -5066,22 +5066,22 @@
         <v>60776708.8</v>
       </c>
       <c r="C28" s="27" t="n">
-        <v>57976102.90415462</v>
+        <v>57981608.29531024</v>
       </c>
       <c r="D28" s="28" t="n">
-        <v>-2800605.895845376</v>
+        <v>-2795100.504689753</v>
       </c>
       <c r="E28" s="29" t="n">
-        <v>-4.608024934455445</v>
+        <v>-4.598966544713183</v>
       </c>
       <c r="F28" s="30" t="n">
         <v>1.888227</v>
       </c>
       <c r="G28" s="30" t="n">
-        <v>1.395811</v>
+        <v>1.396035</v>
       </c>
       <c r="H28" s="31" t="n">
-        <v>-0.4924160000000002</v>
+        <v>-0.4921920000000002</v>
       </c>
       <c r="I28" s="30" t="n">
         <v>1.892367</v>
@@ -5112,10 +5112,10 @@
         <v>3.549869</v>
       </c>
       <c r="G29" s="36" t="n">
-        <v>1.278651</v>
+        <v>1.278772</v>
       </c>
       <c r="H29" s="37" t="n">
-        <v>-2.271218</v>
+        <v>-2.271097</v>
       </c>
       <c r="I29" s="36" t="n">
         <v>3.270644</v>
@@ -5134,28 +5134,28 @@
         <v>96048368.26000001</v>
       </c>
       <c r="C30" s="27" t="n">
-        <v>93416888.58999512</v>
+        <v>93404531.89824064</v>
       </c>
       <c r="D30" s="28" t="n">
-        <v>-2631479.670004889</v>
+        <v>-2643836.361759365</v>
       </c>
       <c r="E30" s="29" t="n">
-        <v>-2.739744274344728</v>
+        <v>-2.752609346368676</v>
       </c>
       <c r="F30" s="30" t="n">
         <v>1.649876</v>
       </c>
       <c r="G30" s="30" t="n">
-        <v>1.393761</v>
+        <v>1.39217</v>
       </c>
       <c r="H30" s="31" t="n">
-        <v>-0.2561149999999999</v>
+        <v>-0.257706</v>
       </c>
       <c r="I30" s="30" t="n">
         <v>1.750748</v>
       </c>
       <c r="J30" s="30" t="n">
-        <v>1.459124</v>
+        <v>1.454767</v>
       </c>
     </row>
     <row r="31"/>
@@ -5228,28 +5228,28 @@
         <v>348203867.78</v>
       </c>
       <c r="C34" s="21" t="n">
-        <v>330169135.8224195</v>
+        <v>329740211.3003739</v>
       </c>
       <c r="D34" s="22" t="n">
-        <v>-18034731.95758045</v>
+        <v>-18463656.47962612</v>
       </c>
       <c r="E34" s="23" t="n">
-        <v>-5.179360031972718</v>
+        <v>-5.302542041632838</v>
       </c>
       <c r="F34" s="24" t="n">
         <v>1.326631</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>1.195777</v>
+        <v>1.192079</v>
       </c>
       <c r="H34" s="25" t="n">
-        <v>-0.1308539999999998</v>
+        <v>-0.1345519999999998</v>
       </c>
       <c r="I34" s="24" t="n">
         <v>1.7402</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>1.343454</v>
+        <v>1.343587</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -5274,10 +5274,10 @@
         <v>0.75745</v>
       </c>
       <c r="G35" s="36" t="n">
-        <v>0.482897</v>
+        <v>0.482828</v>
       </c>
       <c r="H35" s="37" t="n">
-        <v>-0.2745529999999999</v>
+        <v>-0.274622</v>
       </c>
       <c r="I35" s="36" t="n">
         <v>1.304845</v>
@@ -5296,22 +5296,22 @@
         <v>130867992.35</v>
       </c>
       <c r="C36" s="27" t="n">
-        <v>113203592.3140549</v>
+        <v>113190363.893052</v>
       </c>
       <c r="D36" s="28" t="n">
-        <v>-17664400.03594506</v>
+        <v>-17677628.45694798</v>
       </c>
       <c r="E36" s="29" t="n">
-        <v>-13.49787653859814</v>
+        <v>-13.50798475586761</v>
       </c>
       <c r="F36" s="30" t="n">
         <v>2.023419</v>
       </c>
       <c r="G36" s="30" t="n">
-        <v>1.628366</v>
+        <v>1.627147</v>
       </c>
       <c r="H36" s="31" t="n">
-        <v>-0.3950530000000001</v>
+        <v>-0.3962720000000002</v>
       </c>
       <c r="I36" s="30" t="n">
         <v>2.418044</v>
@@ -5330,28 +5330,28 @@
         <v>134942171.49</v>
       </c>
       <c r="C37" s="33" t="n">
-        <v>140663200.6047232</v>
+        <v>140247504.5036805</v>
       </c>
       <c r="D37" s="39" t="n">
-        <v>5721029.114723235</v>
+        <v>5305333.013680518</v>
       </c>
       <c r="E37" s="37" t="n">
-        <v>4.239615423075652</v>
+        <v>3.931560427033497</v>
       </c>
       <c r="F37" s="36" t="n">
         <v>0.994684</v>
       </c>
       <c r="G37" s="36" t="n">
-        <v>1.233614</v>
+        <v>1.226066</v>
       </c>
       <c r="H37" s="35" t="n">
-        <v>0.23893</v>
+        <v>0.2313820000000001</v>
       </c>
       <c r="I37" s="36" t="n">
         <v>1.266873</v>
       </c>
       <c r="J37" s="36" t="n">
-        <v>1.268035</v>
+        <v>1.268363</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -5376,10 +5376,10 @@
         <v>1.234839</v>
       </c>
       <c r="G38" s="30" t="n">
-        <v>0.587283</v>
+        <v>0.5870919999999999</v>
       </c>
       <c r="H38" s="31" t="n">
-        <v>-0.647556</v>
+        <v>-0.6477470000000001</v>
       </c>
       <c r="I38" s="30" t="n">
         <v>1.917953</v>
@@ -5432,22 +5432,22 @@
         <v>60921854.69</v>
       </c>
       <c r="C40" s="27" t="n">
-        <v>54105961.96934212</v>
+        <v>54097767.04882433</v>
       </c>
       <c r="D40" s="28" t="n">
-        <v>-6815892.720657878</v>
+        <v>-6824087.641175672</v>
       </c>
       <c r="E40" s="29" t="n">
-        <v>-11.18792714919868</v>
+        <v>-11.20137867748766</v>
       </c>
       <c r="F40" s="30" t="n">
         <v>2.220508</v>
       </c>
       <c r="G40" s="30" t="n">
-        <v>1.46742</v>
+        <v>1.466473</v>
       </c>
       <c r="H40" s="31" t="n">
-        <v>-0.7530880000000002</v>
+        <v>-0.7540350000000002</v>
       </c>
       <c r="I40" s="30" t="n">
         <v>2.536862</v>
@@ -5466,22 +5466,22 @@
         <v>56234877.77</v>
       </c>
       <c r="C41" s="33" t="n">
-        <v>54152908.32040801</v>
+        <v>54147874.81992287</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>-2081969.449591987</v>
+        <v>-2087002.950077124</v>
       </c>
       <c r="E41" s="35" t="n">
-        <v>-3.702274339613963</v>
+        <v>-3.711225191264649</v>
       </c>
       <c r="F41" s="36" t="n">
         <v>2.008263</v>
       </c>
       <c r="G41" s="36" t="n">
-        <v>1.838641</v>
+        <v>1.837035</v>
       </c>
       <c r="H41" s="37" t="n">
-        <v>-0.1696219999999999</v>
+        <v>-0.1712279999999999</v>
       </c>
       <c r="I41" s="36" t="n">
         <v>2.258991</v>
@@ -5512,10 +5512,10 @@
         <v>1.200174</v>
       </c>
       <c r="G42" s="30" t="n">
-        <v>1.081534</v>
+        <v>1.081533</v>
       </c>
       <c r="H42" s="31" t="n">
-        <v>-0.1186400000000001</v>
+        <v>-0.118641</v>
       </c>
       <c r="I42" s="30" t="n">
         <v>2.510655</v>
@@ -5534,28 +5534,28 @@
         <v>134942171.49</v>
       </c>
       <c r="C43" s="33" t="n">
-        <v>140663200.6047232</v>
+        <v>140247504.5036805</v>
       </c>
       <c r="D43" s="39" t="n">
-        <v>5721029.114723235</v>
+        <v>5305333.013680518</v>
       </c>
       <c r="E43" s="37" t="n">
-        <v>4.239615423075652</v>
+        <v>3.931560427033497</v>
       </c>
       <c r="F43" s="36" t="n">
         <v>0.994684</v>
       </c>
       <c r="G43" s="36" t="n">
-        <v>1.233614</v>
+        <v>1.226066</v>
       </c>
       <c r="H43" s="35" t="n">
-        <v>0.23893</v>
+        <v>0.2313820000000001</v>
       </c>
       <c r="I43" s="36" t="n">
         <v>1.266873</v>
       </c>
       <c r="J43" s="36" t="n">
-        <v>1.268035</v>
+        <v>1.268363</v>
       </c>
     </row>
     <row r="44"/>
@@ -5668,40 +5668,40 @@
         <v>319437971.72</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>290638589.9751463</v>
+        <v>290631738.6745474</v>
       </c>
       <c r="F47" s="22" t="n">
-        <v>-28799381.74485373</v>
+        <v>-28806233.04545259</v>
       </c>
       <c r="G47" s="23" t="n">
-        <v>-9.015641312078429</v>
+        <v>-9.017786110507361</v>
       </c>
       <c r="H47" s="24" t="n">
         <v>1.709876</v>
       </c>
       <c r="I47" s="24" t="n">
-        <v>1.16794</v>
+        <v>1.167463</v>
       </c>
       <c r="J47" s="25" t="n">
-        <v>-0.541936</v>
+        <v>-0.542413</v>
       </c>
       <c r="K47" s="24" t="n">
         <v>58.80500666344847</v>
       </c>
       <c r="L47" s="24" t="n">
-        <v>64.14478055441049</v>
+        <v>64.08550333585117</v>
       </c>
       <c r="M47" s="24" t="n">
         <v>58.34369066429844</v>
       </c>
       <c r="N47" s="24" t="n">
-        <v>63.23251543358717</v>
+        <v>63.15873081972169</v>
       </c>
       <c r="O47" s="24" t="n">
         <v>1.734517</v>
       </c>
       <c r="P47" s="24" t="n">
-        <v>1.17538</v>
+        <v>1.173858</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
@@ -5724,40 +5724,40 @@
         <v>348203867.78</v>
       </c>
       <c r="E48" s="21" t="n">
-        <v>330169135.8224195</v>
+        <v>329740211.3003739</v>
       </c>
       <c r="F48" s="22" t="n">
-        <v>-18034731.95758045</v>
+        <v>-18463656.47962612</v>
       </c>
       <c r="G48" s="23" t="n">
-        <v>-5.179360031972718</v>
+        <v>-5.302542041632838</v>
       </c>
       <c r="H48" s="24" t="n">
         <v>1.326631</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>1.195777</v>
+        <v>1.192079</v>
       </c>
       <c r="J48" s="25" t="n">
-        <v>-0.1308539999999998</v>
+        <v>-0.1345519999999998</v>
       </c>
       <c r="K48" s="24" t="n">
         <v>63.18210218256325</v>
       </c>
       <c r="L48" s="24" t="n">
-        <v>65.76460816985382</v>
+        <v>65.72750787568698</v>
       </c>
       <c r="M48" s="24" t="n">
         <v>62.95956107948448</v>
       </c>
       <c r="N48" s="24" t="n">
-        <v>64.98147837140895</v>
+        <v>64.94301620792133</v>
       </c>
       <c r="O48" s="24" t="n">
         <v>1.7402</v>
       </c>
       <c r="P48" s="24" t="n">
-        <v>1.343454</v>
+        <v>1.343587</v>
       </c>
     </row>
     <row r="49"/>
@@ -5845,25 +5845,25 @@
         </is>
       </c>
       <c r="B53" s="33" t="n">
-        <v>93416888.58999512</v>
+        <v>93404531.89824064</v>
       </c>
       <c r="C53" s="34" t="n">
-        <v>-2631479.670004889</v>
+        <v>-2643836.361759365</v>
       </c>
       <c r="D53" s="35" t="n">
-        <v>-2.739744274344728</v>
+        <v>-2.752609346368676</v>
       </c>
       <c r="E53" s="36" t="n">
-        <v>1.393761</v>
+        <v>1.39217</v>
       </c>
       <c r="F53" s="37" t="n">
-        <v>-0.2561149999999999</v>
+        <v>-0.257706</v>
       </c>
       <c r="G53" s="36" t="n">
-        <v>36.55431518664042</v>
+        <v>36.2526955951482</v>
       </c>
       <c r="H53" s="36" t="n">
-        <v>38.75805218174867</v>
+        <v>38.38019388780192</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
@@ -5873,25 +5873,25 @@
         </is>
       </c>
       <c r="B54" s="27" t="n">
-        <v>57976102.90415462</v>
+        <v>57981608.29531024</v>
       </c>
       <c r="C54" s="28" t="n">
-        <v>-2800605.895845376</v>
+        <v>-2795100.504689753</v>
       </c>
       <c r="D54" s="29" t="n">
-        <v>-4.608024934455445</v>
+        <v>-4.598966544713183</v>
       </c>
       <c r="E54" s="30" t="n">
-        <v>1.395811</v>
+        <v>1.396035</v>
       </c>
       <c r="F54" s="31" t="n">
-        <v>-0.4924160000000002</v>
+        <v>-0.4921920000000002</v>
       </c>
       <c r="G54" s="30" t="n">
-        <v>63.06359510627515</v>
+        <v>63.06011724269709</v>
       </c>
       <c r="H54" s="30" t="n">
-        <v>63.59827485927953</v>
+        <v>63.59479699570146</v>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
@@ -5910,16 +5910,16 @@
         <v>-5.495074989717708</v>
       </c>
       <c r="E55" s="36" t="n">
-        <v>1.132772</v>
+        <v>1.132763</v>
       </c>
       <c r="F55" s="37" t="n">
-        <v>-0.5095210000000001</v>
+        <v>-0.50953</v>
       </c>
       <c r="G55" s="36" t="n">
-        <v>42.89289594139503</v>
+        <v>42.8937558956998</v>
       </c>
       <c r="H55" s="36" t="n">
-        <v>44.04435495359911</v>
+        <v>44.04722146794835</v>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
@@ -5938,10 +5938,10 @@
         <v>-21.34861485171021</v>
       </c>
       <c r="E56" s="30" t="n">
-        <v>0.788784</v>
+        <v>0.788872</v>
       </c>
       <c r="F56" s="31" t="n">
-        <v>-1.275036</v>
+        <v>-1.274948</v>
       </c>
       <c r="G56" s="30" t="n">
         <v>77.25719575296664</v>
@@ -5966,10 +5966,10 @@
         <v>-72.47247222868683</v>
       </c>
       <c r="E57" s="36" t="n">
-        <v>1.278651</v>
+        <v>1.278772</v>
       </c>
       <c r="F57" s="37" t="n">
-        <v>-2.271218</v>
+        <v>-2.271097</v>
       </c>
       <c r="G57" s="36" t="n">
         <v>96.17122789082067</v>
@@ -6035,25 +6035,25 @@
         </is>
       </c>
       <c r="B61" s="33" t="n">
-        <v>140663200.6047232</v>
+        <v>140247504.5036805</v>
       </c>
       <c r="C61" s="39" t="n">
-        <v>5721029.114723235</v>
+        <v>5305333.013680518</v>
       </c>
       <c r="D61" s="37" t="n">
-        <v>4.239615423075652</v>
+        <v>3.931560427033497</v>
       </c>
       <c r="E61" s="36" t="n">
-        <v>1.233614</v>
+        <v>1.226066</v>
       </c>
       <c r="F61" s="35" t="n">
-        <v>0.23893</v>
+        <v>0.2313820000000001</v>
       </c>
       <c r="G61" s="36" t="n">
-        <v>35.40102167503155</v>
+        <v>35.22846653885239</v>
       </c>
       <c r="H61" s="36" t="n">
-        <v>37.27216468097254</v>
+        <v>37.09357097911566</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
@@ -6091,25 +6091,25 @@
         </is>
       </c>
       <c r="B63" s="33" t="n">
-        <v>54152908.32040801</v>
+        <v>54147874.81992287</v>
       </c>
       <c r="C63" s="34" t="n">
-        <v>-2081969.449591987</v>
+        <v>-2087002.950077124</v>
       </c>
       <c r="D63" s="35" t="n">
-        <v>-3.702274339613963</v>
+        <v>-3.711225191264649</v>
       </c>
       <c r="E63" s="36" t="n">
-        <v>1.838641</v>
+        <v>1.837035</v>
       </c>
       <c r="F63" s="37" t="n">
-        <v>-0.1696219999999999</v>
+        <v>-0.1712279999999999</v>
       </c>
       <c r="G63" s="36" t="n">
-        <v>67.23342740231371</v>
+        <v>67.23684640926994</v>
       </c>
       <c r="H63" s="36" t="n">
-        <v>68.40466799513899</v>
+        <v>68.40808700209521</v>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
@@ -6128,10 +6128,10 @@
         <v>-17.96542241671737</v>
       </c>
       <c r="E64" s="30" t="n">
-        <v>0.587283</v>
+        <v>0.5870919999999999</v>
       </c>
       <c r="F64" s="31" t="n">
-        <v>-0.647556</v>
+        <v>-0.6477470000000001</v>
       </c>
       <c r="G64" s="30" t="n">
         <v>79.76761157755884</v>
@@ -6147,25 +6147,25 @@
         </is>
       </c>
       <c r="B65" s="33" t="n">
-        <v>54105961.96934212</v>
+        <v>54097767.04882433</v>
       </c>
       <c r="C65" s="34" t="n">
-        <v>-6815892.720657878</v>
+        <v>-6824087.641175672</v>
       </c>
       <c r="D65" s="35" t="n">
-        <v>-11.18792714919868</v>
+        <v>-11.20137867748766</v>
       </c>
       <c r="E65" s="36" t="n">
-        <v>1.46742</v>
+        <v>1.466473</v>
       </c>
       <c r="F65" s="37" t="n">
-        <v>-0.7530880000000002</v>
+        <v>-0.7540350000000002</v>
       </c>
       <c r="G65" s="36" t="n">
-        <v>47.91292448368614</v>
+        <v>47.92147696350668</v>
       </c>
       <c r="H65" s="36" t="n">
-        <v>49.24947992003167</v>
+        <v>49.25803239985221</v>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
@@ -6184,10 +6184,10 @@
         <v>-63.93677850194405</v>
       </c>
       <c r="E66" s="30" t="n">
-        <v>1.081534</v>
+        <v>1.081533</v>
       </c>
       <c r="F66" s="31" t="n">
-        <v>-0.1186400000000001</v>
+        <v>-0.118641</v>
       </c>
       <c r="G66" s="30" t="n">
         <v>96.61896840592199</v>
@@ -6248,8 +6248,8 @@
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="21" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="20" customWidth="1" min="25" max="25"/>
@@ -6475,7 +6475,7 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>3.273512</v>
+        <v>3.273167</v>
       </c>
       <c r="C6" s="30" t="inlineStr"/>
       <c r="D6" s="30" t="inlineStr"/>
@@ -6502,10 +6502,10 @@
         <v>1.062622149623083</v>
       </c>
       <c r="U6" s="87" t="n">
-        <v>1.582886276694327</v>
+        <v>1.582425541159931</v>
       </c>
       <c r="V6" s="87" t="n">
-        <v>2.042132837382499</v>
+        <v>2.03280802212494</v>
       </c>
       <c r="W6" s="87" t="n">
         <v>1</v>
@@ -6565,7 +6565,7 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.132772</v>
+        <v>1.132763</v>
       </c>
       <c r="C8" s="89" t="n">
         <v>1.230911</v>
@@ -6580,10 +6580,10 @@
         <v>94.50492501028228</v>
       </c>
       <c r="G8" s="89" t="n">
-        <v>42.89289594139503</v>
+        <v>42.8937558956998</v>
       </c>
       <c r="H8" s="89" t="n">
-        <v>44.04435495359911</v>
+        <v>44.04722146794835</v>
       </c>
       <c r="I8" s="90" t="n">
         <v>64916268.49822187</v>
@@ -6592,10 +6592,10 @@
         <v>67939026.01120937</v>
       </c>
       <c r="K8" s="89" t="n">
-        <v>0.8059850000000001</v>
+        <v>0.8060850000000002</v>
       </c>
       <c r="L8" s="89" t="n">
-        <v>1.494475</v>
+        <v>1.4944775</v>
       </c>
       <c r="M8" s="91" t="inlineStr">
         <is>
@@ -6609,13 +6609,13 @@
         <v>1.44652</v>
       </c>
       <c r="P8" s="91" t="n">
-        <v>1.068115416151299</v>
+        <v>1.067770283895112</v>
       </c>
       <c r="Q8" s="91" t="n">
-        <v>1.511150941852545</v>
+        <v>1.51109536781317</v>
       </c>
       <c r="R8" s="91" t="n">
-        <v>0.008977153183907099</v>
+        <v>0.009130349795721301</v>
       </c>
       <c r="S8" s="91" t="n">
         <v>48.7</v>
@@ -6634,7 +6634,7 @@
         </is>
       </c>
       <c r="B9" s="93" t="n">
-        <v>-0.507228</v>
+        <v>-0.5072369999999999</v>
       </c>
       <c r="C9" s="93" t="n">
         <v>-0.4390889999999998</v>
@@ -6855,7 +6855,7 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>3.198803</v>
+        <v>3.201874</v>
       </c>
       <c r="C14" s="30" t="inlineStr"/>
       <c r="D14" s="30" t="inlineStr"/>
@@ -6933,7 +6933,7 @@
         </is>
       </c>
       <c r="B16" s="89" t="n">
-        <v>1.17411</v>
+        <v>1.174227</v>
       </c>
       <c r="C16" s="89" t="n">
         <v>1.291889</v>
@@ -6978,7 +6978,7 @@
         </is>
       </c>
       <c r="B17" s="93" t="n">
-        <v>-0.7719419999999999</v>
+        <v>-0.771825</v>
       </c>
       <c r="C17" s="93" t="inlineStr"/>
       <c r="D17" s="93" t="inlineStr"/>
@@ -7195,7 +7195,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>3.396898</v>
+        <v>3.390912</v>
       </c>
       <c r="C22" s="30" t="inlineStr"/>
       <c r="D22" s="30" t="inlineStr"/>
@@ -7273,7 +7273,7 @@
         </is>
       </c>
       <c r="B24" s="89" t="n">
-        <v>1.101963</v>
+        <v>1.10186</v>
       </c>
       <c r="C24" s="89" t="n">
         <v>1.186074</v>
@@ -7288,10 +7288,10 @@
         <v>98.03437576150657</v>
       </c>
       <c r="G24" s="89" t="n">
-        <v>34.95178320134742</v>
+        <v>34.9535582079214</v>
       </c>
       <c r="H24" s="89" t="n">
-        <v>33.16172659512515</v>
+        <v>33.1676432837051</v>
       </c>
       <c r="I24" s="90" t="inlineStr"/>
       <c r="J24" s="90" t="inlineStr"/>
@@ -7318,7 +7318,7 @@
         </is>
       </c>
       <c r="B25" s="93" t="n">
-        <v>-0.294219</v>
+        <v>-0.294322</v>
       </c>
       <c r="C25" s="93" t="inlineStr"/>
       <c r="D25" s="93" t="inlineStr"/>
@@ -7475,7 +7475,7 @@
         <v>1075745.421039899</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>3.1988</v>
+        <v>3.2019</v>
       </c>
       <c r="D31" s="101" t="n">
         <v>293</v>
@@ -7484,7 +7484,7 @@
         <v>651350.0082414271</v>
       </c>
       <c r="F31" s="30" t="n">
-        <v>3.3969</v>
+        <v>3.3909</v>
       </c>
       <c r="G31" s="101" t="n">
         <v>170</v>
@@ -7493,7 +7493,7 @@
         <v>1727095.429281326</v>
       </c>
       <c r="I31" s="24" t="n">
-        <v>3.273510658395014</v>
+        <v>3.273178720023511</v>
       </c>
       <c r="J31" s="100" t="n">
         <v>463</v>
@@ -7543,7 +7543,7 @@
         <v>28139806.7910399</v>
       </c>
       <c r="C33" s="89" t="n">
-        <v>1.1741</v>
+        <v>1.1742</v>
       </c>
       <c r="D33" s="102" t="n">
         <v>3049</v>
@@ -7552,7 +7552,7 @@
         <v>38249192.23824143</v>
       </c>
       <c r="F33" s="89" t="n">
-        <v>1.102</v>
+        <v>1.1019</v>
       </c>
       <c r="G33" s="102" t="n">
         <v>3056</v>
@@ -7561,7 +7561,7 @@
         <v>66388999.02928133</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>1.132788888648086</v>
+        <v>1.132774294719232</v>
       </c>
       <c r="J33" s="100" t="n">
         <v>6105</v>
@@ -7653,7 +7653,7 @@
         <v>1.0941</v>
       </c>
       <c r="C40" s="103" t="n">
-        <v>3.1988</v>
+        <v>3.2019</v>
       </c>
       <c r="D40" s="103" t="n">
         <v>7.4996</v>
@@ -7669,7 +7669,7 @@
         <v>1.0619</v>
       </c>
       <c r="C41" s="103" t="n">
-        <v>3.3969</v>
+        <v>3.3909</v>
       </c>
       <c r="D41" s="103" t="n">
         <v>10.0881</v>
@@ -7824,13 +7824,13 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>13.084955</v>
+        <v>13.201532</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>372928.5293421224</v>
+        <v>364733.6088243293</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>0.6121424425434255</v>
+        <v>0.5986909142544513</v>
       </c>
       <c r="E6" s="30" t="inlineStr"/>
       <c r="F6" s="30" t="inlineStr"/>
@@ -7872,19 +7872,19 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.46742</v>
+        <v>1.466473</v>
       </c>
       <c r="C8" s="90" t="n">
-        <v>54105961.96934212</v>
+        <v>54097767.04882433</v>
       </c>
       <c r="D8" s="89" t="n">
-        <v>88.81207285080131</v>
+        <v>88.79862132251235</v>
       </c>
       <c r="E8" s="89" t="n">
-        <v>47.91292448368614</v>
+        <v>47.92147696350669</v>
       </c>
       <c r="F8" s="89" t="n">
-        <v>49.24947992003167</v>
+        <v>49.25803239985221</v>
       </c>
       <c r="G8" s="89" t="n">
         <v>0.390384</v>
@@ -7989,7 +7989,7 @@
         </is>
       </c>
       <c r="B13" s="36" t="n">
-        <v>15.36955</v>
+        <v>15.205382</v>
       </c>
       <c r="C13" s="33" t="n">
         <v>314556.2625889373</v>
@@ -8037,7 +8037,7 @@
         </is>
       </c>
       <c r="B15" s="89" t="n">
-        <v>2.026401</v>
+        <v>2.024248</v>
       </c>
       <c r="C15" s="90" t="n">
         <v>23266815.55258894</v>
@@ -8068,7 +8068,7 @@
         </is>
       </c>
       <c r="B16" s="93" t="n">
-        <v>-1.324451</v>
+        <v>-1.326604</v>
       </c>
       <c r="C16" s="94" t="n">
         <v>-5164620.507411063</v>
@@ -8175,13 +8175,13 @@
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>0.773737</v>
+        <v>0.639619</v>
       </c>
       <c r="C21" s="33" t="n">
-        <v>58372.26675318514</v>
+        <v>50177.34623539197</v>
       </c>
       <c r="D21" s="36" t="n">
-        <v>0.1796599404209805</v>
+        <v>0.1544373644636907</v>
       </c>
       <c r="E21" s="36" t="inlineStr"/>
       <c r="F21" s="36" t="inlineStr"/>
@@ -8223,19 +8223,19 @@
         </is>
       </c>
       <c r="B23" s="89" t="n">
-        <v>1.044238</v>
+        <v>1.044096</v>
       </c>
       <c r="C23" s="90" t="n">
-        <v>30839146.41675318</v>
+        <v>30830951.49623539</v>
       </c>
       <c r="D23" s="89" t="n">
-        <v>94.91766409029242</v>
+        <v>94.89244151433512</v>
       </c>
       <c r="E23" s="89" t="n">
-        <v>36.49011065491852</v>
+        <v>36.51011889672182</v>
       </c>
       <c r="F23" s="89" t="n">
-        <v>35.1934346692729</v>
+        <v>35.21344291107619</v>
       </c>
       <c r="G23" s="89" t="n">
         <v>0.189164</v>
@@ -8254,13 +8254,13 @@
         </is>
       </c>
       <c r="B24" s="93" t="n">
-        <v>-0.1849190000000001</v>
+        <v>-0.1850610000000001</v>
       </c>
       <c r="C24" s="94" t="n">
-        <v>-1651272.213246815</v>
+        <v>-1659467.13376461</v>
       </c>
       <c r="D24" s="93" t="n">
-        <v>-5.082335909707591</v>
+        <v>-5.107558485664886</v>
       </c>
       <c r="E24" s="93" t="inlineStr"/>
       <c r="F24" s="93" t="inlineStr"/>
@@ -8371,16 +8371,16 @@
         <v>116</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>58372.26675318514</v>
+        <v>50177.34623539197</v>
       </c>
       <c r="E30" s="101" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>372928.5293421224</v>
+        <v>364733.6088243293</v>
       </c>
       <c r="G30" s="100" t="n">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -8421,16 +8421,16 @@
         <v>2488</v>
       </c>
       <c r="D32" s="90" t="n">
-        <v>30839146.41675318</v>
+        <v>30830951.49623539</v>
       </c>
       <c r="E32" s="102" t="n">
-        <v>2374</v>
+        <v>2370</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>54105961.96934213</v>
+        <v>54097767.04882433</v>
       </c>
       <c r="G32" s="100" t="n">
-        <v>4862</v>
+        <v>4858</v>
       </c>
     </row>
     <row r="35">
@@ -8481,7 +8481,7 @@
         <v>30780774.15</v>
       </c>
       <c r="C37" s="103" t="n">
-        <v>58372.26675318514</v>
+        <v>50177.34623539197</v>
       </c>
       <c r="D37" s="103" t="n">
         <v>1709644.48</v>
@@ -8526,16 +8526,16 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
@@ -8762,15 +8762,15 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>3.498209</v>
+        <v>3.498402</v>
       </c>
       <c r="C6" s="30" t="inlineStr"/>
       <c r="D6" s="30" t="inlineStr"/>
       <c r="E6" s="27" t="n">
-        <v>7834515.154154621</v>
+        <v>7840020.545310241</v>
       </c>
       <c r="F6" s="30" t="n">
-        <v>12.89065385217868</v>
+        <v>12.89971224192094</v>
       </c>
       <c r="G6" s="30" t="inlineStr"/>
       <c r="H6" s="30" t="inlineStr"/>
@@ -8786,13 +8786,13 @@
       <c r="R6" s="87" t="inlineStr"/>
       <c r="S6" s="87" t="inlineStr"/>
       <c r="T6" s="87" t="n">
-        <v>1.31990978846603</v>
+        <v>1.319909728867453</v>
       </c>
       <c r="U6" s="87" t="n">
-        <v>2.068626184237245</v>
+        <v>2.068848534097421</v>
       </c>
       <c r="V6" s="87" t="n">
-        <v>2.386552467043298</v>
+        <v>2.386536609787511</v>
       </c>
       <c r="W6" s="87" t="n">
         <v>1</v>
@@ -8852,7 +8852,7 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.395811</v>
+        <v>1.396035</v>
       </c>
       <c r="C8" s="89" t="n">
         <v>1.139222</v>
@@ -8861,28 +8861,28 @@
         <v>0.596216</v>
       </c>
       <c r="E8" s="90" t="n">
-        <v>57976102.90415462</v>
+        <v>57981608.29531024</v>
       </c>
       <c r="F8" s="89" t="n">
-        <v>95.39197506554456</v>
+        <v>95.40103345528679</v>
       </c>
       <c r="G8" s="89" t="n">
-        <v>63.06359510627515</v>
+        <v>63.06011724269709</v>
       </c>
       <c r="H8" s="89" t="n">
-        <v>63.59827485927953</v>
+        <v>63.59479699570146</v>
       </c>
       <c r="I8" s="90" t="n">
-        <v>56588884.28851959</v>
+        <v>56586933.8070816</v>
       </c>
       <c r="J8" s="90" t="n">
-        <v>59440198.26908033</v>
+        <v>59449089.47579665</v>
       </c>
       <c r="K8" s="89" t="n">
-        <v>1.12229</v>
+        <v>1.1230675</v>
       </c>
       <c r="L8" s="89" t="n">
-        <v>1.7085775</v>
+        <v>1.7083925</v>
       </c>
       <c r="M8" s="91" t="inlineStr">
         <is>
@@ -8896,16 +8896,16 @@
         <v>1.430505</v>
       </c>
       <c r="P8" s="91" t="n">
-        <v>1.321460688261341</v>
+        <v>1.33191500346878</v>
       </c>
       <c r="Q8" s="91" t="n">
-        <v>1.399551174418131</v>
+        <v>1.399600988689973</v>
       </c>
       <c r="R8" s="91" t="n">
-        <v>0.0089701949613968</v>
+        <v>0.0057776270358176</v>
       </c>
       <c r="S8" s="91" t="n">
-        <v>96.59999999999999</v>
+        <v>96.3</v>
       </c>
       <c r="T8" s="91" t="inlineStr"/>
       <c r="U8" s="91" t="inlineStr"/>
@@ -8921,7 +8921,7 @@
         </is>
       </c>
       <c r="B9" s="93" t="n">
-        <v>-0.494189</v>
+        <v>-0.493965</v>
       </c>
       <c r="C9" s="93" t="n">
         <v>-0.7507779999999999</v>
@@ -8930,10 +8930,10 @@
         <v>-0.383784</v>
       </c>
       <c r="E9" s="94" t="n">
-        <v>-2800605.895845376</v>
+        <v>-2795100.504689753</v>
       </c>
       <c r="F9" s="93" t="n">
-        <v>-4.608024934455445</v>
+        <v>-4.598966544713183</v>
       </c>
       <c r="G9" s="93" t="inlineStr"/>
       <c r="H9" s="93" t="inlineStr"/>
@@ -9142,7 +9142,7 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>3.349419</v>
+        <v>3.347927</v>
       </c>
       <c r="C14" s="30" t="inlineStr"/>
       <c r="D14" s="30" t="inlineStr"/>
@@ -9220,7 +9220,7 @@
         </is>
       </c>
       <c r="B16" s="89" t="n">
-        <v>1.770971</v>
+        <v>1.770741</v>
       </c>
       <c r="C16" s="89" t="n">
         <v>1.286117</v>
@@ -9265,7 +9265,7 @@
         </is>
       </c>
       <c r="B17" s="93" t="n">
-        <v>-0.720604</v>
+        <v>-0.7208340000000002</v>
       </c>
       <c r="C17" s="93" t="inlineStr"/>
       <c r="D17" s="93" t="inlineStr"/>
@@ -9482,15 +9482,15 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>3.649216</v>
+        <v>3.650904</v>
       </c>
       <c r="C22" s="30" t="inlineStr"/>
       <c r="D22" s="30" t="inlineStr"/>
       <c r="E22" s="27" t="n">
-        <v>3888294.438428414</v>
+        <v>3893799.829584033</v>
       </c>
       <c r="F22" s="30" t="n">
-        <v>12.29465657745403</v>
+        <v>12.31206443960406</v>
       </c>
       <c r="G22" s="30" t="inlineStr"/>
       <c r="H22" s="30" t="inlineStr"/>
@@ -9560,7 +9560,7 @@
         </is>
       </c>
       <c r="B24" s="89" t="n">
-        <v>1.102082</v>
+        <v>1.102711</v>
       </c>
       <c r="C24" s="89" t="n">
         <v>1.028476</v>
@@ -9569,16 +9569,16 @@
         <v>0.417533</v>
       </c>
       <c r="E24" s="90" t="n">
-        <v>32510081.11842841</v>
+        <v>32515586.50958403</v>
       </c>
       <c r="F24" s="89" t="n">
-        <v>102.795785912191</v>
+        <v>102.813193774341</v>
       </c>
       <c r="G24" s="89" t="n">
-        <v>54.37655557368799</v>
+        <v>54.36845689609257</v>
       </c>
       <c r="H24" s="89" t="n">
-        <v>52.52826186426815</v>
+        <v>52.52016318667273</v>
       </c>
       <c r="I24" s="90" t="inlineStr"/>
       <c r="J24" s="90" t="inlineStr"/>
@@ -9605,15 +9605,15 @@
         </is>
       </c>
       <c r="B25" s="93" t="n">
-        <v>-0.229433</v>
+        <v>-0.228804</v>
       </c>
       <c r="C25" s="93" t="inlineStr"/>
       <c r="D25" s="93" t="inlineStr"/>
       <c r="E25" s="94" t="n">
-        <v>884192.148428414</v>
+        <v>889697.5395840332</v>
       </c>
       <c r="F25" s="93" t="n">
-        <v>2.795785912190958</v>
+        <v>2.813193774340988</v>
       </c>
       <c r="G25" s="93" t="inlineStr"/>
       <c r="H25" s="93" t="inlineStr"/>
@@ -9762,28 +9762,28 @@
         <v>3946220.715726208</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>3.3494</v>
+        <v>3.3479</v>
       </c>
       <c r="D31" s="101" t="n">
         <v>1093</v>
       </c>
       <c r="E31" s="27" t="n">
-        <v>3888294.438428414</v>
+        <v>3893799.829584033</v>
       </c>
       <c r="F31" s="30" t="n">
-        <v>3.6492</v>
+        <v>3.6509</v>
       </c>
       <c r="G31" s="101" t="n">
-        <v>989</v>
+        <v>992</v>
       </c>
       <c r="H31" s="21" t="n">
-        <v>7834515.154154621</v>
+        <v>7840020.545310241</v>
       </c>
       <c r="I31" s="24" t="n">
-        <v>3.498191680110883</v>
+        <v>3.498387022520587</v>
       </c>
       <c r="J31" s="100" t="n">
-        <v>2082</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -9830,28 +9830,28 @@
         <v>25466021.78572621</v>
       </c>
       <c r="C33" s="89" t="n">
-        <v>1.771</v>
+        <v>1.7707</v>
       </c>
       <c r="D33" s="102" t="n">
         <v>3207</v>
       </c>
       <c r="E33" s="90" t="n">
-        <v>32510081.11842841</v>
+        <v>32515586.50958403</v>
       </c>
       <c r="F33" s="89" t="n">
-        <v>1.1021</v>
+        <v>1.1027</v>
       </c>
       <c r="G33" s="102" t="n">
-        <v>3218</v>
+        <v>3221</v>
       </c>
       <c r="H33" s="21" t="n">
-        <v>57976102.90415462</v>
+        <v>57981608.29531024</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>1.395834137070398</v>
+        <v>1.396011266236857</v>
       </c>
       <c r="J33" s="100" t="n">
-        <v>6425</v>
+        <v>6428</v>
       </c>
     </row>
     <row r="36">
@@ -9902,7 +9902,7 @@
         <v>28621786.68</v>
       </c>
       <c r="C38" s="103" t="n">
-        <v>3888294.438428414</v>
+        <v>3893799.829584033</v>
       </c>
       <c r="D38" s="103" t="n">
         <v>3004102.29</v>
@@ -9940,7 +9940,7 @@
         <v>1.4839</v>
       </c>
       <c r="C40" s="103" t="n">
-        <v>3.3494</v>
+        <v>3.3479</v>
       </c>
       <c r="D40" s="103" t="n">
         <v>5.3264</v>
@@ -9956,7 +9956,7 @@
         <v>0.7589</v>
       </c>
       <c r="C41" s="103" t="n">
-        <v>3.6492</v>
+        <v>3.6509</v>
       </c>
       <c r="D41" s="103" t="n">
         <v>6.8233</v>
@@ -10111,13 +10111,13 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>2.113019</v>
+        <v>2.074638</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>2290245.590408013</v>
+        <v>2285212.089922875</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>4.07264260407054</v>
+        <v>4.063691752419853</v>
       </c>
       <c r="E6" s="30" t="inlineStr"/>
       <c r="F6" s="30" t="inlineStr"/>
@@ -10159,19 +10159,19 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.838641</v>
+        <v>1.837035</v>
       </c>
       <c r="C8" s="90" t="n">
-        <v>54152908.32040801</v>
+        <v>54147874.81992287</v>
       </c>
       <c r="D8" s="89" t="n">
-        <v>96.29772566038604</v>
+        <v>96.28877480873535</v>
       </c>
       <c r="E8" s="89" t="n">
-        <v>67.23342740231371</v>
+        <v>67.23684640926994</v>
       </c>
       <c r="F8" s="89" t="n">
-        <v>68.40466799513899</v>
+        <v>68.40808700209521</v>
       </c>
       <c r="G8" s="89" t="n">
         <v>0.5269430000000001</v>
@@ -10451,10 +10451,10 @@
       </c>
       <c r="B21" s="36" t="inlineStr"/>
       <c r="C21" s="33" t="n">
-        <v>1508287.953333751</v>
+        <v>1503254.452848613</v>
       </c>
       <c r="D21" s="36" t="n">
-        <v>5.013706013188887</v>
+        <v>4.996974134111059</v>
       </c>
       <c r="E21" s="36" t="inlineStr"/>
       <c r="F21" s="36" t="inlineStr"/>
@@ -10497,16 +10497,16 @@
       </c>
       <c r="B23" s="89" t="inlineStr"/>
       <c r="C23" s="90" t="n">
-        <v>30691442.66333375</v>
+        <v>30686409.16284861</v>
       </c>
       <c r="D23" s="89" t="n">
-        <v>102.0215472081998</v>
+        <v>102.004815329122</v>
       </c>
       <c r="E23" s="89" t="n">
-        <v>55.54124364953076</v>
+        <v>55.55043933568512</v>
       </c>
       <c r="F23" s="89" t="n">
-        <v>53.74671562325757</v>
+        <v>53.75591130941192</v>
       </c>
       <c r="G23" s="89" t="inlineStr"/>
       <c r="H23" s="89" t="inlineStr"/>
@@ -10520,10 +10520,10 @@
       </c>
       <c r="B24" s="93" t="inlineStr"/>
       <c r="C24" s="94" t="n">
-        <v>608148.0033337511</v>
+        <v>603114.502848614</v>
       </c>
       <c r="D24" s="93" t="n">
-        <v>2.021547208199805</v>
+        <v>2.00481532912198</v>
       </c>
       <c r="E24" s="93" t="inlineStr"/>
       <c r="F24" s="93" t="inlineStr"/>
@@ -10634,16 +10634,16 @@
         <v>279</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>1508287.953333751</v>
+        <v>1503254.452848613</v>
       </c>
       <c r="E30" s="101" t="n">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>2290245.590408013</v>
+        <v>2285212.089922875</v>
       </c>
       <c r="G30" s="100" t="n">
-        <v>603</v>
+        <v>600</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -10684,16 +10684,16 @@
         <v>2582</v>
       </c>
       <c r="D32" s="90" t="n">
-        <v>30691442.66333375</v>
+        <v>30686409.16284861</v>
       </c>
       <c r="E32" s="102" t="n">
-        <v>2655</v>
+        <v>2652</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>54152908.32040802</v>
+        <v>54147874.81992288</v>
       </c>
       <c r="G32" s="100" t="n">
-        <v>5237</v>
+        <v>5234</v>
       </c>
     </row>
     <row r="35">
@@ -10744,7 +10744,7 @@
         <v>29183154.71</v>
       </c>
       <c r="C37" s="103" t="n">
-        <v>1508287.953333751</v>
+        <v>1503254.452848613</v>
       </c>
       <c r="D37" s="103" t="n">
         <v>900139.95</v>
@@ -10789,12 +10789,12 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="20" customWidth="1" min="20" max="20"/>
@@ -11025,7 +11025,7 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>1.731119</v>
+        <v>1.73327</v>
       </c>
       <c r="C6" s="30" t="inlineStr"/>
       <c r="D6" s="30" t="inlineStr"/>
@@ -11049,13 +11049,13 @@
       <c r="R6" s="87" t="inlineStr"/>
       <c r="S6" s="87" t="inlineStr"/>
       <c r="T6" s="87" t="n">
-        <v>1.96387320954858</v>
+        <v>1.963873210933244</v>
       </c>
       <c r="U6" s="87" t="n">
-        <v>2.385943629481712</v>
+        <v>2.386211717282722</v>
       </c>
       <c r="V6" s="87" t="n">
-        <v>2.488307061062233</v>
+        <v>2.48757717338841</v>
       </c>
       <c r="W6" s="87" t="n">
         <v>1</v>
@@ -11115,7 +11115,7 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.278651</v>
+        <v>1.278772</v>
       </c>
       <c r="C8" s="89" t="n">
         <v>1.679734</v>
@@ -11142,10 +11142,10 @@
         <v>5028155.559131417</v>
       </c>
       <c r="K8" s="89" t="n">
-        <v>0.0954975</v>
+        <v>0.0955975</v>
       </c>
       <c r="L8" s="89" t="n">
-        <v>2.847329999999999</v>
+        <v>2.8475275</v>
       </c>
       <c r="M8" s="91" t="inlineStr">
         <is>
@@ -11159,13 +11159,13 @@
         <v>2.9111225</v>
       </c>
       <c r="P8" s="91" t="n">
-        <v>0.0047252674846294</v>
+        <v>0.0047849978879831</v>
       </c>
       <c r="Q8" s="91" t="n">
-        <v>1.39793455058691</v>
+        <v>1.397426180492488</v>
       </c>
       <c r="R8" s="91" t="n">
-        <v>0.4343072400950868</v>
+        <v>0.4339204200430258</v>
       </c>
       <c r="S8" s="91" t="n">
         <v>94.5</v>
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="B9" s="93" t="n">
-        <v>-2.271349</v>
+        <v>-2.271228</v>
       </c>
       <c r="C9" s="93" t="n">
         <v>-1.590266</v>
@@ -11405,7 +11405,7 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>1.592167</v>
+        <v>1.593061</v>
       </c>
       <c r="C14" s="30" t="inlineStr"/>
       <c r="D14" s="30" t="inlineStr"/>
@@ -11483,7 +11483,7 @@
         </is>
       </c>
       <c r="B16" s="89" t="n">
-        <v>0.071755</v>
+        <v>0.071795</v>
       </c>
       <c r="C16" s="89" t="n">
         <v>0</v>
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="B17" s="93" t="n">
-        <v>-3.524756</v>
+        <v>-3.524716</v>
       </c>
       <c r="C17" s="93" t="inlineStr"/>
       <c r="D17" s="93" t="inlineStr"/>
@@ -11745,7 +11745,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>1.763586</v>
+        <v>1.766032</v>
       </c>
       <c r="C22" s="30" t="inlineStr"/>
       <c r="D22" s="30" t="inlineStr"/>
@@ -11823,7 +11823,7 @@
         </is>
       </c>
       <c r="B24" s="89" t="n">
-        <v>1.65378</v>
+        <v>1.653926</v>
       </c>
       <c r="C24" s="89" t="n">
         <v>2.204923</v>
@@ -11868,7 +11868,7 @@
         </is>
       </c>
       <c r="B25" s="93" t="n">
-        <v>-1.859683</v>
+        <v>-1.859537</v>
       </c>
       <c r="C25" s="93" t="inlineStr"/>
       <c r="D25" s="93" t="inlineStr"/>
@@ -12025,7 +12025,7 @@
         <v>48042.49059439893</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>1.5922</v>
+        <v>1.5931</v>
       </c>
       <c r="D31" s="101" t="n">
         <v>14</v>
@@ -12034,7 +12034,7 @@
         <v>205607.1637863073</v>
       </c>
       <c r="F31" s="30" t="n">
-        <v>1.7636</v>
+        <v>1.766</v>
       </c>
       <c r="G31" s="101" t="n">
         <v>62</v>
@@ -12043,7 +12043,7 @@
         <v>253649.6543807063</v>
       </c>
       <c r="I31" s="24" t="n">
-        <v>1.731135997996982</v>
+        <v>1.733251890628228</v>
       </c>
       <c r="J31" s="100" t="n">
         <v>76</v>
@@ -12102,7 +12102,7 @@
         <v>3420873.393786307</v>
       </c>
       <c r="F33" s="89" t="n">
-        <v>1.6538</v>
+        <v>1.6539</v>
       </c>
       <c r="G33" s="102" t="n">
         <v>319</v>
@@ -12111,7 +12111,7 @@
         <v>4509479.984380705</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>1.278676896186332</v>
+        <v>1.278753184232867</v>
       </c>
       <c r="J33" s="100" t="n">
         <v>415</v>
@@ -12203,7 +12203,7 @@
         <v>0</v>
       </c>
       <c r="C40" s="103" t="n">
-        <v>1.5922</v>
+        <v>1.5931</v>
       </c>
       <c r="D40" s="103" t="n">
         <v>4.1846</v>
@@ -12219,7 +12219,7 @@
         <v>1.6468</v>
       </c>
       <c r="C41" s="103" t="n">
-        <v>1.7636</v>
+        <v>1.766</v>
       </c>
       <c r="D41" s="103" t="n">
         <v>4.5073</v>
@@ -12374,7 +12374,7 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>0.264223</v>
+        <v>0.263407</v>
       </c>
       <c r="C6" s="27" t="n">
         <v>9632.854304801946</v>
@@ -12422,7 +12422,7 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.081534</v>
+        <v>1.081533</v>
       </c>
       <c r="C8" s="90" t="n">
         <v>4944722.024304802</v>
@@ -12723,7 +12723,7 @@
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>0.264223</v>
+        <v>0.263407</v>
       </c>
       <c r="C21" s="33" t="n">
         <v>9632.854304801946</v>
@@ -12771,7 +12771,7 @@
         </is>
       </c>
       <c r="B23" s="89" t="n">
-        <v>0.8788319999999999</v>
+        <v>0.878831</v>
       </c>
       <c r="C23" s="90" t="n">
         <v>4242612.144304802</v>
@@ -12802,7 +12802,7 @@
         </is>
       </c>
       <c r="B24" s="93" t="n">
-        <v>0.260366</v>
+        <v>0.2603650000000001</v>
       </c>
       <c r="C24" s="94" t="n">
         <v>-3917204.555695198</v>
@@ -13073,8 +13073,8 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
@@ -13083,7 +13083,7 @@
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
@@ -13310,15 +13310,15 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>6.58134</v>
+        <v>6.471549</v>
       </c>
       <c r="C6" s="30" t="inlineStr"/>
       <c r="D6" s="30" t="inlineStr"/>
       <c r="E6" s="27" t="n">
-        <v>801220.3299951135</v>
+        <v>845102.408240634</v>
       </c>
       <c r="F6" s="30" t="n">
-        <v>0.834184218336989</v>
+        <v>0.8798716975107455</v>
       </c>
       <c r="G6" s="30" t="inlineStr"/>
       <c r="H6" s="30" t="inlineStr"/>
@@ -13337,10 +13337,10 @@
         <v>1.063919377060216</v>
       </c>
       <c r="U6" s="87" t="n">
-        <v>1.577815603114244</v>
+        <v>1.576137044489517</v>
       </c>
       <c r="V6" s="87" t="n">
-        <v>1.671814117715265</v>
+        <v>1.644727981446204</v>
       </c>
       <c r="W6" s="87" t="n">
         <v>1</v>
@@ -13359,19 +13359,19 @@
         </is>
       </c>
       <c r="B7" s="36" t="n">
-        <v>9.707261000000001</v>
+        <v>9.616255000000001</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>9.401413</v>
+        <v>9.362686</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>6.140176</v>
+        <v>5.932962</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>3432700</v>
+        <v>3488938.77</v>
       </c>
       <c r="F7" s="36" t="n">
-        <v>3.573928492681714</v>
+        <v>3.632481043879422</v>
       </c>
       <c r="G7" s="36" t="inlineStr"/>
       <c r="H7" s="36" t="inlineStr"/>
@@ -13400,37 +13400,37 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.393761</v>
+        <v>1.39217</v>
       </c>
       <c r="C8" s="89" t="n">
-        <v>1.459124</v>
+        <v>1.454767</v>
       </c>
       <c r="D8" s="89" t="n">
-        <v>0.922764</v>
+        <v>0.9260429999999999</v>
       </c>
       <c r="E8" s="90" t="n">
-        <v>93416888.58999512</v>
+        <v>93404531.89824064</v>
       </c>
       <c r="F8" s="89" t="n">
-        <v>97.26025572565528</v>
+        <v>97.24739065363131</v>
       </c>
       <c r="G8" s="89" t="n">
-        <v>36.55431518664042</v>
+        <v>36.25269559514821</v>
       </c>
       <c r="H8" s="89" t="n">
-        <v>38.75805218174867</v>
+        <v>38.38019388780192</v>
       </c>
       <c r="I8" s="90" t="n">
-        <v>92002127.05520062</v>
+        <v>91939670.69338544</v>
       </c>
       <c r="J8" s="90" t="n">
-        <v>94703020.7379773</v>
+        <v>94721039.55187429</v>
       </c>
       <c r="K8" s="89" t="n">
-        <v>1.1073875</v>
+        <v>1.1014475</v>
       </c>
       <c r="L8" s="89" t="n">
-        <v>1.6963375</v>
+        <v>1.69725</v>
       </c>
       <c r="M8" s="91" t="inlineStr">
         <is>
@@ -13438,22 +13438,22 @@
         </is>
       </c>
       <c r="N8" s="91" t="n">
-        <v>1.0611</v>
+        <v>1.0491925</v>
       </c>
       <c r="O8" s="91" t="n">
-        <v>1.655505</v>
+        <v>1.65149</v>
       </c>
       <c r="P8" s="91" t="n">
-        <v>1.321221786339621</v>
+        <v>1.321242654772142</v>
       </c>
       <c r="Q8" s="91" t="n">
-        <v>1.399549055411368</v>
+        <v>1.399551694404155</v>
       </c>
       <c r="R8" s="91" t="n">
-        <v>0.009279802438067501</v>
+        <v>0.009113370538041499</v>
       </c>
       <c r="S8" s="91" t="n">
-        <v>95.5</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="T8" s="91" t="inlineStr"/>
       <c r="U8" s="91" t="inlineStr"/>
@@ -13469,19 +13469,19 @@
         </is>
       </c>
       <c r="B9" s="93" t="n">
-        <v>-0.2562389999999999</v>
+        <v>-0.25783</v>
       </c>
       <c r="C9" s="93" t="n">
-        <v>-0.2908759999999999</v>
+        <v>-0.2952330000000001</v>
       </c>
       <c r="D9" s="93" t="n">
-        <v>-0.187236</v>
+        <v>-0.1839570000000001</v>
       </c>
       <c r="E9" s="94" t="n">
-        <v>-2631479.670004889</v>
+        <v>-2643836.361759365</v>
       </c>
       <c r="F9" s="93" t="n">
-        <v>-2.739744274344728</v>
+        <v>-2.752609346368676</v>
       </c>
       <c r="G9" s="93" t="inlineStr"/>
       <c r="H9" s="93" t="inlineStr"/>
@@ -13690,15 +13690,15 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>7.128517</v>
+        <v>6.114163</v>
       </c>
       <c r="C14" s="30" t="inlineStr"/>
       <c r="D14" s="30" t="inlineStr"/>
       <c r="E14" s="27" t="n">
-        <v>338307.7662979924</v>
+        <v>104711.7669209058</v>
       </c>
       <c r="F14" s="30" t="n">
-        <v>0.8886435902117895</v>
+        <v>0.2750496730011545</v>
       </c>
       <c r="G14" s="30" t="inlineStr"/>
       <c r="H14" s="30" t="inlineStr"/>
@@ -13727,19 +13727,19 @@
         </is>
       </c>
       <c r="B15" s="36" t="n">
-        <v>10.6597</v>
+        <v>9.392632000000001</v>
       </c>
       <c r="C15" s="36" t="n">
-        <v>10.450559</v>
+        <v>9.254704</v>
       </c>
       <c r="D15" s="36" t="n">
-        <v>6.903143</v>
+        <v>6.191567</v>
       </c>
       <c r="E15" s="33" t="n">
-        <v>2395186</v>
+        <v>3005953.77</v>
       </c>
       <c r="F15" s="36" t="n">
-        <v>6.291509974944509</v>
+        <v>7.895832777987619</v>
       </c>
       <c r="G15" s="36" t="inlineStr"/>
       <c r="H15" s="36" t="inlineStr"/>
@@ -13768,25 +13768,25 @@
         </is>
       </c>
       <c r="B16" s="89" t="n">
-        <v>1.806487</v>
+        <v>1.719657</v>
       </c>
       <c r="C16" s="89" t="n">
-        <v>1.63323</v>
+        <v>1.572304</v>
       </c>
       <c r="D16" s="89" t="n">
-        <v>1.185057</v>
+        <v>1.141956</v>
       </c>
       <c r="E16" s="90" t="n">
-        <v>36013251.34629799</v>
+        <v>35168887.5769209</v>
       </c>
       <c r="F16" s="89" t="n">
-        <v>94.59713361526728</v>
+        <v>92.37921689501354</v>
       </c>
       <c r="G16" s="89" t="n">
-        <v>40.6375909811354</v>
+        <v>41.7355256853764</v>
       </c>
       <c r="H16" s="89" t="n">
-        <v>45.78712577653809</v>
+        <v>46.81880209293997</v>
       </c>
       <c r="I16" s="90" t="inlineStr"/>
       <c r="J16" s="90" t="inlineStr"/>
@@ -13813,15 +13813,15 @@
         </is>
       </c>
       <c r="B17" s="93" t="n">
-        <v>-0.5117719999999999</v>
+        <v>-0.5986019999999999</v>
       </c>
       <c r="C17" s="93" t="inlineStr"/>
       <c r="D17" s="93" t="inlineStr"/>
       <c r="E17" s="94" t="n">
-        <v>-2056878.233702004</v>
+        <v>-2901242.003079094</v>
       </c>
       <c r="F17" s="93" t="n">
-        <v>-5.40286638473271</v>
+        <v>-7.620783104986462</v>
       </c>
       <c r="G17" s="93" t="inlineStr"/>
       <c r="H17" s="93" t="inlineStr"/>
@@ -14030,15 +14030,15 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>6.18145</v>
+        <v>6.522093</v>
       </c>
       <c r="C22" s="30" t="inlineStr"/>
       <c r="D22" s="30" t="inlineStr"/>
       <c r="E22" s="27" t="n">
-        <v>462912.563697121</v>
+        <v>740390.6413197282</v>
       </c>
       <c r="F22" s="30" t="n">
-        <v>0.7984246749061834</v>
+        <v>1.277014718239675</v>
       </c>
       <c r="G22" s="30" t="inlineStr"/>
       <c r="H22" s="30" t="inlineStr"/>
@@ -14067,19 +14067,19 @@
         </is>
       </c>
       <c r="B23" s="36" t="n">
-        <v>7.493368</v>
+        <v>11.033229</v>
       </c>
       <c r="C23" s="36" t="n">
-        <v>7.028147</v>
+        <v>10.062559</v>
       </c>
       <c r="D23" s="36" t="n">
-        <v>4.388129</v>
+        <v>4.293936</v>
       </c>
       <c r="E23" s="33" t="n">
-        <v>1037514</v>
+        <v>482985</v>
       </c>
       <c r="F23" s="36" t="n">
-        <v>1.78948864888146</v>
+        <v>0.8330453132006045</v>
       </c>
       <c r="G23" s="36" t="inlineStr"/>
       <c r="H23" s="36" t="inlineStr"/>
@@ -14108,25 +14108,25 @@
         </is>
       </c>
       <c r="B24" s="89" t="n">
-        <v>1.132182</v>
+        <v>1.19248</v>
       </c>
       <c r="C24" s="89" t="n">
-        <v>1.346532</v>
+        <v>1.380946</v>
       </c>
       <c r="D24" s="89" t="n">
-        <v>0.756445</v>
+        <v>0.792906</v>
       </c>
       <c r="E24" s="90" t="n">
-        <v>57403637.24369712</v>
+        <v>58235644.32131973</v>
       </c>
       <c r="F24" s="89" t="n">
-        <v>99.00893602602471</v>
+        <v>100.4439694050391</v>
       </c>
       <c r="G24" s="89" t="n">
-        <v>33.33850251549081</v>
+        <v>31.93465406053349</v>
       </c>
       <c r="H24" s="89" t="n">
-        <v>33.22225566194423</v>
+        <v>31.73430843731733</v>
       </c>
       <c r="I24" s="90" t="inlineStr"/>
       <c r="J24" s="90" t="inlineStr"/>
@@ -14153,15 +14153,15 @@
         </is>
       </c>
       <c r="B25" s="93" t="n">
-        <v>-0.07425100000000007</v>
+        <v>-0.0139530000000001</v>
       </c>
       <c r="C25" s="93" t="inlineStr"/>
       <c r="D25" s="93" t="inlineStr"/>
       <c r="E25" s="94" t="n">
-        <v>-574601.436302878</v>
+        <v>257405.6413197294</v>
       </c>
       <c r="F25" s="93" t="n">
-        <v>-0.9910639739752749</v>
+        <v>0.4439694050390725</v>
       </c>
       <c r="G25" s="93" t="inlineStr"/>
       <c r="H25" s="93" t="inlineStr"/>
@@ -14273,31 +14273,31 @@
         </is>
       </c>
       <c r="B30" s="33" t="n">
-        <v>35674943.58</v>
+        <v>35064175.81</v>
       </c>
       <c r="C30" s="36" t="n">
-        <v>1.7565</v>
+        <v>1.7067</v>
       </c>
       <c r="D30" s="99" t="n">
-        <v>3797</v>
+        <v>3717</v>
       </c>
       <c r="E30" s="33" t="n">
-        <v>56940724.68</v>
+        <v>57495253.68</v>
       </c>
       <c r="F30" s="36" t="n">
-        <v>1.0911</v>
+        <v>1.1239</v>
       </c>
       <c r="G30" s="99" t="n">
-        <v>5104</v>
+        <v>5158</v>
       </c>
       <c r="H30" s="21" t="n">
-        <v>92615668.25999999</v>
+        <v>92559429.49000001</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>1.349028369774802</v>
+        <v>1.3460104803822</v>
       </c>
       <c r="J30" s="100" t="n">
-        <v>8901</v>
+        <v>8875</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -14307,31 +14307,31 @@
         </is>
       </c>
       <c r="B31" s="27" t="n">
-        <v>338307.7662979924</v>
+        <v>104711.7669209058</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>7.1285</v>
+        <v>6.1142</v>
       </c>
       <c r="D31" s="101" t="n">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="E31" s="27" t="n">
-        <v>462912.563697121</v>
+        <v>740390.6413197282</v>
       </c>
       <c r="F31" s="30" t="n">
-        <v>6.1815</v>
+        <v>6.5221</v>
       </c>
       <c r="G31" s="101" t="n">
-        <v>152</v>
+        <v>232</v>
       </c>
       <c r="H31" s="21" t="n">
-        <v>801220.3299951134</v>
+        <v>845102.408240634</v>
       </c>
       <c r="I31" s="24" t="n">
-        <v>6.581361864071963</v>
+        <v>6.471559462769775</v>
       </c>
       <c r="J31" s="100" t="n">
-        <v>246</v>
+        <v>263</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -14341,31 +14341,31 @@
         </is>
       </c>
       <c r="B32" s="33" t="n">
-        <v>2395186</v>
+        <v>3005953.77</v>
       </c>
       <c r="C32" s="36" t="n">
-        <v>10.6597</v>
+        <v>9.3926</v>
       </c>
       <c r="D32" s="99" t="n">
-        <v>311</v>
+        <v>391</v>
       </c>
       <c r="E32" s="33" t="n">
-        <v>1037514</v>
+        <v>482985</v>
       </c>
       <c r="F32" s="36" t="n">
-        <v>7.4934</v>
+        <v>11.0332</v>
       </c>
       <c r="G32" s="99" t="n">
-        <v>126</v>
+        <v>72</v>
       </c>
       <c r="H32" s="21" t="n">
-        <v>3432700</v>
+        <v>3488938.77</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>9.707270384413338</v>
+        <v>9.616223839193356</v>
       </c>
       <c r="J32" s="100" t="n">
-        <v>437</v>
+        <v>463</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -14375,31 +14375,31 @@
         </is>
       </c>
       <c r="B33" s="90" t="n">
-        <v>36013251.34629799</v>
+        <v>35168887.57692091</v>
       </c>
       <c r="C33" s="89" t="n">
-        <v>1.8065</v>
+        <v>1.7197</v>
       </c>
       <c r="D33" s="102" t="n">
-        <v>3891</v>
+        <v>3748</v>
       </c>
       <c r="E33" s="90" t="n">
-        <v>57403637.24369712</v>
+        <v>58235644.32131973</v>
       </c>
       <c r="F33" s="89" t="n">
-        <v>1.1322</v>
+        <v>1.1925</v>
       </c>
       <c r="G33" s="102" t="n">
-        <v>5256</v>
+        <v>5390</v>
       </c>
       <c r="H33" s="21" t="n">
-        <v>93416888.58999512</v>
+        <v>93404531.89824064</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>1.39377760911004</v>
+        <v>1.392198812117355</v>
       </c>
       <c r="J33" s="100" t="n">
-        <v>9147</v>
+        <v>9138</v>
       </c>
     </row>
     <row r="36">
@@ -14431,13 +14431,13 @@
         </is>
       </c>
       <c r="B37" s="103" t="n">
-        <v>35674943.58</v>
+        <v>35064175.81</v>
       </c>
       <c r="C37" s="103" t="n">
-        <v>338307.7662979924</v>
+        <v>104711.7669209058</v>
       </c>
       <c r="D37" s="103" t="n">
-        <v>2395186</v>
+        <v>3005953.77</v>
       </c>
     </row>
     <row r="38">
@@ -14447,13 +14447,13 @@
         </is>
       </c>
       <c r="B38" s="103" t="n">
-        <v>56940724.68</v>
+        <v>57495253.68</v>
       </c>
       <c r="C38" s="103" t="n">
-        <v>462912.563697121</v>
+        <v>740390.6413197282</v>
       </c>
       <c r="D38" s="103" t="n">
-        <v>1037514</v>
+        <v>482985</v>
       </c>
     </row>
     <row r="39">
@@ -14485,13 +14485,13 @@
         </is>
       </c>
       <c r="B40" s="103" t="n">
-        <v>1.7565</v>
+        <v>1.7067</v>
       </c>
       <c r="C40" s="103" t="n">
-        <v>7.1285</v>
+        <v>6.1142</v>
       </c>
       <c r="D40" s="103" t="n">
-        <v>10.6597</v>
+        <v>9.3926</v>
       </c>
     </row>
     <row r="41">
@@ -14501,13 +14501,13 @@
         </is>
       </c>
       <c r="B41" s="103" t="n">
-        <v>1.0911</v>
+        <v>1.1239</v>
       </c>
       <c r="C41" s="103" t="n">
-        <v>6.1815</v>
+        <v>6.5221</v>
       </c>
       <c r="D41" s="103" t="n">
-        <v>7.4934</v>
+        <v>11.0332</v>
       </c>
     </row>
   </sheetData>
@@ -14659,13 +14659,13 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>6.788014</v>
+        <v>6.868838</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>5970096.83472322</v>
+        <v>5627705.543680534</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>4.42418909433782</v>
+        <v>4.170457227374305</v>
       </c>
       <c r="E6" s="30" t="inlineStr"/>
       <c r="F6" s="30" t="inlineStr"/>
@@ -14680,13 +14680,13 @@
         </is>
       </c>
       <c r="B7" s="36" t="n">
-        <v>2.491331</v>
+        <v>1.077915</v>
       </c>
       <c r="C7" s="33" t="n">
-        <v>249067.72</v>
+        <v>322372.5300000001</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>0.1845736712621801</v>
+        <v>0.2388968003407961</v>
       </c>
       <c r="E7" s="36" t="inlineStr"/>
       <c r="F7" s="36" t="inlineStr"/>
@@ -14707,28 +14707,28 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>1.233614</v>
+        <v>1.226066</v>
       </c>
       <c r="C8" s="90" t="n">
-        <v>140663200.6047232</v>
+        <v>140247504.5036805</v>
       </c>
       <c r="D8" s="89" t="n">
-        <v>104.2396154230756</v>
+        <v>103.9315604270335</v>
       </c>
       <c r="E8" s="89" t="n">
-        <v>35.40102167503155</v>
+        <v>35.22846653885239</v>
       </c>
       <c r="F8" s="89" t="n">
-        <v>37.27216468097254</v>
+        <v>37.09357097911566</v>
       </c>
       <c r="G8" s="89" t="n">
-        <v>0.237734</v>
+        <v>0.237884</v>
       </c>
       <c r="H8" s="89" t="n">
-        <v>1.268035</v>
+        <v>1.268363</v>
       </c>
       <c r="I8" s="89" t="n">
-        <v>0.801245</v>
+        <v>0.8016529999999999</v>
       </c>
     </row>
     <row r="9"/>
@@ -14824,13 +14824,13 @@
         </is>
       </c>
       <c r="B13" s="36" t="n">
-        <v>7.160565</v>
+        <v>7.625158</v>
       </c>
       <c r="C13" s="33" t="n">
-        <v>3513675.409218004</v>
+        <v>2230397.544401558</v>
       </c>
       <c r="D13" s="36" t="n">
-        <v>7.963153144508721</v>
+        <v>5.05482013865323</v>
       </c>
       <c r="E13" s="36" t="inlineStr"/>
       <c r="F13" s="36" t="inlineStr"/>
@@ -14845,20 +14845,22 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>5.986453</v>
+        <v>2.156944</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>53447</v>
+        <v>148251.81</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>0.1211286179133091</v>
+        <v>0.3359877420331636</v>
       </c>
       <c r="E14" s="30" t="inlineStr"/>
       <c r="F14" s="30" t="inlineStr"/>
       <c r="G14" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="30" t="inlineStr"/>
+      <c r="H14" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I14" s="30" t="n">
         <v>0</v>
       </c>
@@ -14870,28 +14872,28 @@
         </is>
       </c>
       <c r="B15" s="89" t="n">
-        <v>1.747051</v>
+        <v>1.625541</v>
       </c>
       <c r="C15" s="90" t="n">
-        <v>47584400.64921801</v>
+        <v>46206317.97440156</v>
       </c>
       <c r="D15" s="89" t="n">
-        <v>107.8420245265954</v>
+        <v>104.7188323966201</v>
       </c>
       <c r="E15" s="89" t="n">
-        <v>40.6262353912885</v>
+        <v>42.0545748898078</v>
       </c>
       <c r="F15" s="89" t="n">
-        <v>44.90122644053605</v>
+        <v>46.33537904732218</v>
       </c>
       <c r="G15" s="89" t="n">
-        <v>0.373304</v>
+        <v>0.374003</v>
       </c>
       <c r="H15" s="89" t="n">
-        <v>1.833878</v>
+        <v>1.835166</v>
       </c>
       <c r="I15" s="89" t="n">
-        <v>1.104193</v>
+        <v>1.10583</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -14901,13 +14903,13 @@
         </is>
       </c>
       <c r="B16" s="93" t="n">
-        <v>0.4158769999999998</v>
+        <v>0.2943669999999998</v>
       </c>
       <c r="C16" s="94" t="n">
-        <v>3460228.409218006</v>
+        <v>2082145.734401554</v>
       </c>
       <c r="D16" s="93" t="n">
-        <v>7.842024526595416</v>
+        <v>4.718832396620057</v>
       </c>
       <c r="E16" s="93" t="inlineStr"/>
       <c r="F16" s="93" t="inlineStr"/>
@@ -15008,13 +15010,13 @@
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>6.255116</v>
+        <v>6.3723</v>
       </c>
       <c r="C21" s="33" t="n">
-        <v>2456421.425505216</v>
+        <v>3397307.999278976</v>
       </c>
       <c r="D21" s="36" t="n">
-        <v>2.70477377369136</v>
+        <v>3.740787098741305</v>
       </c>
       <c r="E21" s="36" t="inlineStr"/>
       <c r="F21" s="36" t="inlineStr"/>
@@ -15029,13 +15031,13 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>1.547208</v>
+        <v>0.171171</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>195620.7199999999</v>
+        <v>174120.7199999999</v>
       </c>
       <c r="D22" s="30" t="n">
-        <v>0.2153986231974824</v>
+        <v>0.1917249019334677</v>
       </c>
       <c r="E22" s="30" t="inlineStr"/>
       <c r="F22" s="30" t="inlineStr"/>
@@ -15056,19 +15058,19 @@
         </is>
       </c>
       <c r="B23" s="89" t="n">
-        <v>0.969357</v>
+        <v>1.028305</v>
       </c>
       <c r="C23" s="90" t="n">
-        <v>93078799.95550522</v>
+        <v>94041186.52927898</v>
       </c>
       <c r="D23" s="89" t="n">
-        <v>102.4893751504939</v>
+        <v>103.5490621968079</v>
       </c>
       <c r="E23" s="89" t="n">
-        <v>31.12343018393726</v>
+        <v>29.64031175994104</v>
       </c>
       <c r="F23" s="89" t="n">
-        <v>31.02667666079664</v>
+        <v>29.52781736565282</v>
       </c>
       <c r="G23" s="89" t="n">
         <v>0.168985</v>
@@ -15087,13 +15089,13 @@
         </is>
       </c>
       <c r="B24" s="93" t="n">
-        <v>0.1394770000000001</v>
+        <v>0.1984250000000001</v>
       </c>
       <c r="C24" s="94" t="n">
-        <v>2260800.705505222</v>
+        <v>3223187.279278979</v>
       </c>
       <c r="D24" s="93" t="n">
-        <v>2.489375150493884</v>
+        <v>3.549062196807841</v>
       </c>
       <c r="E24" s="93" t="inlineStr"/>
       <c r="F24" s="93" t="inlineStr"/>
@@ -15173,22 +15175,22 @@
         </is>
       </c>
       <c r="B29" s="33" t="n">
-        <v>44070725.24</v>
+        <v>43975920.42999999</v>
       </c>
       <c r="C29" s="99" t="n">
-        <v>4483</v>
+        <v>4468</v>
       </c>
       <c r="D29" s="33" t="n">
-        <v>90622378.53</v>
+        <v>90643878.53</v>
       </c>
       <c r="E29" s="99" t="n">
-        <v>7832</v>
+        <v>7834</v>
       </c>
       <c r="F29" s="21" t="n">
-        <v>134693103.77</v>
+        <v>134619798.96</v>
       </c>
       <c r="G29" s="100" t="n">
-        <v>12315</v>
+        <v>12302</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -15198,22 +15200,22 @@
         </is>
       </c>
       <c r="B30" s="27" t="n">
-        <v>3513675.409218004</v>
+        <v>2230397.544401558</v>
       </c>
       <c r="C30" s="101" t="n">
-        <v>1044</v>
+        <v>695</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>2456421.425505216</v>
+        <v>3397307.999278976</v>
       </c>
       <c r="E30" s="101" t="n">
-        <v>888</v>
+        <v>1177</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>5970096.83472322</v>
+        <v>5627705.543680534</v>
       </c>
       <c r="G30" s="100" t="n">
-        <v>1932</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -15223,22 +15225,22 @@
         </is>
       </c>
       <c r="B31" s="33" t="n">
-        <v>53447</v>
+        <v>148251.81</v>
       </c>
       <c r="C31" s="99" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D31" s="33" t="n">
-        <v>195620.7199999999</v>
+        <v>174120.7199999999</v>
       </c>
       <c r="E31" s="99" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F31" s="21" t="n">
-        <v>249067.7199999999</v>
+        <v>322372.5299999999</v>
       </c>
       <c r="G31" s="100" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -15248,22 +15250,22 @@
         </is>
       </c>
       <c r="B32" s="90" t="n">
-        <v>47584400.64921801</v>
+        <v>46206317.97440155</v>
       </c>
       <c r="C32" s="102" t="n">
-        <v>5527</v>
+        <v>5163</v>
       </c>
       <c r="D32" s="90" t="n">
-        <v>93078799.95550522</v>
+        <v>94041186.52927898</v>
       </c>
       <c r="E32" s="102" t="n">
-        <v>8720</v>
+        <v>9011</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>140663200.6047232</v>
+        <v>140247504.5036805</v>
       </c>
       <c r="G32" s="100" t="n">
-        <v>14247</v>
+        <v>14174</v>
       </c>
     </row>
     <row r="35">
@@ -15295,13 +15297,13 @@
         </is>
       </c>
       <c r="B36" s="103" t="n">
-        <v>44070725.24</v>
+        <v>43975920.42999999</v>
       </c>
       <c r="C36" s="103" t="n">
-        <v>3513675.409218004</v>
+        <v>2230397.544401558</v>
       </c>
       <c r="D36" s="103" t="n">
-        <v>53447</v>
+        <v>148251.81</v>
       </c>
     </row>
     <row r="37">
@@ -15311,13 +15313,13 @@
         </is>
       </c>
       <c r="B37" s="103" t="n">
-        <v>90622378.53</v>
+        <v>90643878.53</v>
       </c>
       <c r="C37" s="103" t="n">
-        <v>2456421.425505216</v>
+        <v>3397307.999278976</v>
       </c>
       <c r="D37" s="103" t="n">
-        <v>195620.7199999999</v>
+        <v>174120.7199999999</v>
       </c>
     </row>
   </sheetData>
@@ -15449,7 +15451,7 @@
       </c>
       <c r="C11" s="44" t="inlineStr">
         <is>
-          <t>The optimizer scores 1,494 candidate accept/reject policies — only monotone ones (a better score is never rejected while a worse one is accepted) — and keeps the efficient frontier: for each level of risk, the maximum attainable production.</t>
+          <t>The optimizer scores 1,495 candidate accept/reject policies — only monotone ones (a better score is never rejected while a worse one is accepted) — and keeps the efficient frontier: for each level of risk, the maximum attainable production.</t>
         </is>
       </c>
     </row>
@@ -15628,7 +15630,7 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>20260908T080239Z_8554dd50756a  ·  git 8554dd50756a (dirty)  ·  cfg 541c2ee33624</t>
+          <t>20260908T125042Z_73da737810a7  ·  git 73da737810a7 (dirty)  ·  cfg 541c2ee33624</t>
         </is>
       </c>
     </row>
@@ -16351,7 +16353,7 @@
         <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7887999999999999</v>
+        <v>0.7889</v>
       </c>
       <c r="E7" t="n">
         <v>0.4817</v>
@@ -16476,10 +16478,10 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0.7543</v>
+        <v>0.7541</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7321</v>
+        <v>0.7318</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -16510,7 +16512,7 @@
         <v>40</v>
       </c>
       <c r="D10" t="n">
-        <v>1.3958</v>
+        <v>1.396</v>
       </c>
       <c r="E10" t="n">
         <v>1.07</v>
@@ -16529,10 +16531,10 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0.5094</v>
+        <v>0.5095</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4898</v>
+        <v>0.4897</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -16563,7 +16565,7 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>1.2787</v>
+        <v>1.2788</v>
       </c>
       <c r="E11" t="n">
         <v>1.2516</v>
@@ -16616,29 +16618,29 @@
         <v>67</v>
       </c>
       <c r="D12" t="n">
-        <v>1.3938</v>
+        <v>1.3922</v>
       </c>
       <c r="E12" t="n">
-        <v>1.3491</v>
+        <v>1.346</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[1.0551, 1.6839]</t>
+          <t>[1.0354, 1.6854]</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1.2203</v>
+        <v>1.2205</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[0.8502, 1.6127]</t>
+          <t>[0.8623, 1.5701]</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>0.8971</v>
+        <v>0.8992</v>
       </c>
       <c r="J12" t="n">
-        <v>0.902</v>
+        <v>0.9026999999999999</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -23403,17 +23405,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="AO53" s="65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="AP53" s="68" t="inlineStr">
+      <c r="AO53" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="AP53" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AQ53" s="82" t="inlineStr">
+      <c r="AQ53" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -23601,27 +23603,27 @@
           <t>R</t>
         </is>
       </c>
-      <c r="AM54" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AN54" s="65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="AO54" s="71" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="AP54" s="71" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="AQ54" s="66" t="inlineStr">
+      <c r="AM54" s="65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AN54" s="67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AO54" s="67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AP54" s="67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AQ54" s="84" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -23809,7 +23811,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="AM55" s="65" t="inlineStr">
+      <c r="AM55" s="70" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -28172,12 +28174,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="K87" s="65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L87" s="67" t="inlineStr">
+      <c r="K87" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="L87" s="65" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -28370,17 +28372,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="I88" s="65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J88" s="67" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K88" s="71" t="inlineStr">
+      <c r="I88" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J88" s="65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K88" s="67" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -28578,12 +28580,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="I89" s="70" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J89" s="71" t="inlineStr">
+      <c r="I89" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J89" s="70" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -28781,17 +28783,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="H90" s="65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I90" s="71" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J90" s="71" t="inlineStr">
+      <c r="H90" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I90" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J90" s="70" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -28989,12 +28991,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="H91" s="70" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I91" s="71" t="inlineStr">
+      <c r="H91" s="60" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I91" s="65" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -29197,7 +29199,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="H92" s="70" t="inlineStr">
+      <c r="H92" s="65" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -29280,17 +29282,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="Z92" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AA92" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AB92" s="65" t="inlineStr">
+      <c r="Z92" s="65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA92" s="67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AB92" s="67" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -29488,17 +29490,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="Z93" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AA93" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AB93" s="70" t="inlineStr">
+      <c r="Z93" s="70" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA93" s="71" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AB93" s="71" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -29696,17 +29698,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="Z94" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AA94" s="60" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="AB94" s="73" t="inlineStr">
+      <c r="Z94" s="73" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA94" s="74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AB94" s="74" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -29840,7 +29842,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
@@ -29849,9 +29851,9 @@
     <col width="21" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="20" customWidth="1" min="25" max="25"/>
@@ -30077,7 +30079,7 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>2.598018</v>
+        <v>2.598623</v>
       </c>
       <c r="C6" s="30" t="inlineStr"/>
       <c r="D6" s="30" t="inlineStr"/>
@@ -30101,13 +30103,13 @@
       <c r="R6" s="87" t="inlineStr"/>
       <c r="S6" s="87" t="inlineStr"/>
       <c r="T6" s="87" t="n">
-        <v>1.42551882423777</v>
+        <v>1.425518816277971</v>
       </c>
       <c r="U6" s="87" t="n">
-        <v>2.201300449740799</v>
+        <v>2.201800385926937</v>
       </c>
       <c r="V6" s="87" t="n">
-        <v>2.400769307466525</v>
+        <v>2.400644627883875</v>
       </c>
       <c r="W6" s="87" t="n">
         <v>1</v>
@@ -30167,7 +30169,7 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>0.788784</v>
+        <v>0.788872</v>
       </c>
       <c r="C8" s="89" t="n">
         <v>0.610657</v>
@@ -30194,10 +30196,10 @@
         <v>29231314.52245024</v>
       </c>
       <c r="K8" s="89" t="n">
-        <v>0.409655</v>
+        <v>0.4096600000000001</v>
       </c>
       <c r="L8" s="89" t="n">
-        <v>1.36873</v>
+        <v>1.3688325</v>
       </c>
       <c r="M8" s="91" t="inlineStr">
         <is>
@@ -30211,13 +30213,13 @@
         <v>1.171635</v>
       </c>
       <c r="P8" s="91" t="n">
-        <v>0.1972230806819833</v>
+        <v>0.1971421427294327</v>
       </c>
       <c r="Q8" s="91" t="n">
-        <v>0.7994666183804098</v>
+        <v>0.7995452804723839</v>
       </c>
       <c r="R8" s="91" t="n">
-        <v>0.1310334694239029</v>
+        <v>0.1310402082192714</v>
       </c>
       <c r="S8" s="91" t="n">
         <v>95.90000000000001</v>
@@ -30236,7 +30238,7 @@
         </is>
       </c>
       <c r="B9" s="93" t="n">
-        <v>-1.271216</v>
+        <v>-1.271128</v>
       </c>
       <c r="C9" s="93" t="n">
         <v>-1.299343</v>
@@ -30457,7 +30459,7 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>2.411543</v>
+        <v>2.415169</v>
       </c>
       <c r="C14" s="30" t="inlineStr"/>
       <c r="D14" s="30" t="inlineStr"/>
@@ -30535,7 +30537,7 @@
         </is>
       </c>
       <c r="B16" s="89" t="n">
-        <v>0.877795</v>
+        <v>0.878562</v>
       </c>
       <c r="C16" s="89" t="n">
         <v>0.289817</v>
@@ -30580,7 +30582,7 @@
         </is>
       </c>
       <c r="B17" s="93" t="n">
-        <v>-1.964049</v>
+        <v>-1.963282</v>
       </c>
       <c r="C17" s="93" t="inlineStr"/>
       <c r="D17" s="93" t="inlineStr"/>
@@ -30797,7 +30799,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>2.670886</v>
+        <v>2.670311</v>
       </c>
       <c r="C22" s="30" t="inlineStr"/>
       <c r="D22" s="30" t="inlineStr"/>
@@ -30875,7 +30877,7 @@
         </is>
       </c>
       <c r="B24" s="89" t="n">
-        <v>0.767539</v>
+        <v>0.767465</v>
       </c>
       <c r="C24" s="89" t="n">
         <v>0.6827220000000001</v>
@@ -30920,7 +30922,7 @@
         </is>
       </c>
       <c r="B25" s="93" t="n">
-        <v>-0.8988689999999999</v>
+        <v>-0.8989429999999999</v>
       </c>
       <c r="C25" s="93" t="inlineStr"/>
       <c r="D25" s="93" t="inlineStr"/>
@@ -31077,7 +31079,7 @@
         <v>1159035.412193135</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>2.4115</v>
+        <v>2.4152</v>
       </c>
       <c r="D31" s="101" t="n">
         <v>221</v>
@@ -31086,7 +31088,7 @@
         <v>2966051.055141377</v>
       </c>
       <c r="F31" s="30" t="n">
-        <v>2.6709</v>
+        <v>2.6703</v>
       </c>
       <c r="G31" s="101" t="n">
         <v>399</v>
@@ -31095,7 +31097,7 @@
         <v>4125086.467334512</v>
       </c>
       <c r="I31" s="24" t="n">
-        <v>2.598015761498893</v>
+        <v>2.598623942784763</v>
       </c>
       <c r="J31" s="100" t="n">
         <v>620</v>
@@ -31145,7 +31147,7 @@
         <v>5403714.412193135</v>
       </c>
       <c r="C33" s="89" t="n">
-        <v>0.8778</v>
+        <v>0.8786</v>
       </c>
       <c r="D33" s="102" t="n">
         <v>498</v>
@@ -31163,7 +31165,7 @@
         <v>28127768.46733451</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>0.7887534334270999</v>
+        <v>0.7889075834428904</v>
       </c>
       <c r="J33" s="100" t="n">
         <v>1767</v>
@@ -31255,7 +31257,7 @@
         <v>0.4661</v>
       </c>
       <c r="C40" s="103" t="n">
-        <v>2.4115</v>
+        <v>2.4152</v>
       </c>
       <c r="D40" s="103" t="n">
         <v>4.1311</v>
@@ -31271,7 +31273,7 @@
         <v>0.485</v>
       </c>
       <c r="C41" s="103" t="n">
-        <v>2.6709</v>
+        <v>2.6703</v>
       </c>
       <c r="D41" s="103" t="n">
         <v>7.4951</v>
@@ -31426,7 +31428,7 @@
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>0.856851</v>
+        <v>0.853596</v>
       </c>
       <c r="C6" s="27" t="n">
         <v>1670080.713641318</v>
@@ -31474,7 +31476,7 @@
         </is>
       </c>
       <c r="B8" s="89" t="n">
-        <v>0.587283</v>
+        <v>0.5870919999999999</v>
       </c>
       <c r="C8" s="90" t="n">
         <v>27814666.30364132</v>
@@ -31591,7 +31593,7 @@
         </is>
       </c>
       <c r="B13" s="36" t="n">
-        <v>1.750371</v>
+        <v>1.743467</v>
       </c>
       <c r="C13" s="33" t="n">
         <v>11723.44647764834</v>
@@ -31639,7 +31641,7 @@
         </is>
       </c>
       <c r="B15" s="89" t="n">
-        <v>0.334914</v>
+        <v>0.334902</v>
       </c>
       <c r="C15" s="90" t="n">
         <v>6302875.906477649</v>
@@ -31670,7 +31672,7 @@
         </is>
       </c>
       <c r="B16" s="93" t="n">
-        <v>-1.335787</v>
+        <v>-1.335799</v>
       </c>
       <c r="C16" s="94" t="n">
         <v>-5772838.493522352</v>
@@ -31777,7 +31779,7 @@
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>0.850535</v>
+        <v>0.847305</v>
       </c>
       <c r="C21" s="33" t="n">
         <v>1658357.26716367</v>
@@ -31825,7 +31827,7 @@
         </is>
       </c>
       <c r="B23" s="89" t="n">
-        <v>0.660403</v>
+        <v>0.660161</v>
       </c>
       <c r="C23" s="90" t="n">
         <v>21511790.39716367</v>
@@ -31856,7 +31858,7 @@
         </is>
       </c>
       <c r="B24" s="93" t="n">
-        <v>-0.334983</v>
+        <v>-0.335225</v>
       </c>
       <c r="C24" s="94" t="n">
         <v>-318522.5428363271</v>
@@ -33229,7 +33231,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -33502,7 +33504,7 @@
         </is>
       </c>
       <c r="B13" s="36" t="n">
-        <v>2.584612</v>
+        <v>2.60128</v>
       </c>
       <c r="C13" s="33" t="n">
         <v>4855951.690037477</v>
@@ -33542,7 +33544,7 @@
         </is>
       </c>
       <c r="B15" s="89" t="n">
-        <v>1.749533</v>
+        <v>1.754429</v>
       </c>
       <c r="C15" s="90" t="n">
         <v>16250265.38003748</v>
@@ -33571,7 +33573,7 @@
         </is>
       </c>
       <c r="B16" s="93" t="n">
-        <v>0.3473550000000001</v>
+        <v>0.3522510000000001</v>
       </c>
       <c r="C16" s="94" t="n">
         <v>4855951.690037476</v>
@@ -33676,7 +33678,7 @@
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>1.446014</v>
+        <v>1.458385</v>
       </c>
       <c r="C21" s="33" t="n">
         <v>3769826.724763093</v>
@@ -33716,7 +33718,7 @@
         </is>
       </c>
       <c r="B23" s="89" t="n">
-        <v>0.240899</v>
+        <v>0.242019</v>
       </c>
       <c r="C23" s="90" t="n">
         <v>40863189.6347631</v>
@@ -33745,7 +33747,7 @@
         </is>
       </c>
       <c r="B24" s="93" t="n">
-        <v>0.119966</v>
+        <v>0.121086</v>
       </c>
       <c r="C24" s="94" t="n">
         <v>3769826.724763095</v>

</xml_diff>